<commit_message>
feat: Update active ETF holdings for 2026-06-17 (29 ETFs/1645 rows), daily stock total (21 sheets/15518 rows)
</commit_message>
<xml_diff>
--- a/wiki/金融投資/高股息ETF持股明細.xlsx
+++ b/wiki/金融投資/高股息ETF持股明細.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -37,9 +37,6 @@
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -2253,11 +2250,11 @@
         <v>11948</v>
       </c>
       <c r="H2" s="6">
-        <f>G2-F2</f>
+        <f t="shared" ref="H2:H33" si="0">G2-F2</f>
         <v>4368</v>
       </c>
       <c r="I2" s="11">
-        <f>IF(F2=0,0,H2/F2)</f>
+        <f t="shared" ref="I2:I33" si="1">IF(F2=0,0,H2/F2)</f>
         <v>0.57625329815303428</v>
       </c>
     </row>
@@ -2284,11 +2281,11 @@
         <v>33440</v>
       </c>
       <c r="H3" s="16">
-        <f>G3-F3</f>
+        <f t="shared" si="0"/>
         <v>11109</v>
       </c>
       <c r="I3" s="11">
-        <f>IF(F3=0,0,H3/F3)</f>
+        <f t="shared" si="1"/>
         <v>0.49746988491334915</v>
       </c>
     </row>
@@ -2315,11 +2312,11 @@
         <v>13060</v>
       </c>
       <c r="H4" s="6">
-        <f>G4-F4</f>
+        <f t="shared" si="0"/>
         <v>3244</v>
       </c>
       <c r="I4" s="11">
-        <f>IF(F4=0,0,H4/F4)</f>
+        <f t="shared" si="1"/>
         <v>0.33048084759576202</v>
       </c>
     </row>
@@ -2346,11 +2343,11 @@
         <v>162670</v>
       </c>
       <c r="H5" s="16">
-        <f>G5-F5</f>
+        <f t="shared" si="0"/>
         <v>39570</v>
       </c>
       <c r="I5" s="11">
-        <f>IF(F5=0,0,H5/F5)</f>
+        <f t="shared" si="1"/>
         <v>0.3214459788789602</v>
       </c>
       <c r="J5" s="12"/>
@@ -2378,11 +2375,11 @@
         <v>75070</v>
       </c>
       <c r="H6" s="16">
-        <f>G6-F6</f>
+        <f t="shared" si="0"/>
         <v>17850</v>
       </c>
       <c r="I6" s="11">
-        <f>IF(F6=0,0,H6/F6)</f>
+        <f t="shared" si="1"/>
         <v>0.31195386228591404</v>
       </c>
     </row>
@@ -2409,11 +2406,11 @@
         <v>63910</v>
       </c>
       <c r="H7" s="16">
-        <f>G7-F7</f>
+        <f t="shared" si="0"/>
         <v>14870</v>
       </c>
       <c r="I7" s="11">
-        <f>IF(F7=0,0,H7/F7)</f>
+        <f t="shared" si="1"/>
         <v>0.30322185970636217</v>
       </c>
     </row>
@@ -2440,11 +2437,11 @@
         <v>203680</v>
       </c>
       <c r="H8" s="16">
-        <f>G8-F8</f>
+        <f t="shared" si="0"/>
         <v>46940</v>
       </c>
       <c r="I8" s="11">
-        <f>IF(F8=0,0,H8/F8)</f>
+        <f t="shared" si="1"/>
         <v>0.29947684062779123</v>
       </c>
     </row>
@@ -2471,11 +2468,11 @@
         <v>68460</v>
       </c>
       <c r="H9" s="16">
-        <f>G9-F9</f>
+        <f t="shared" si="0"/>
         <v>15760</v>
       </c>
       <c r="I9" s="11">
-        <f>IF(F9=0,0,H9/F9)</f>
+        <f t="shared" si="1"/>
         <v>0.29905123339658446</v>
       </c>
     </row>
@@ -2502,11 +2499,11 @@
         <v>116010</v>
       </c>
       <c r="H10" s="16">
-        <f>G10-F10</f>
+        <f t="shared" si="0"/>
         <v>26570</v>
       </c>
       <c r="I10" s="11">
-        <f>IF(F10=0,0,H10/F10)</f>
+        <f t="shared" si="1"/>
         <v>0.29707066189624332</v>
       </c>
     </row>
@@ -2533,11 +2530,11 @@
         <v>27490</v>
       </c>
       <c r="H11" s="6">
-        <f>G11-F11</f>
+        <f t="shared" si="0"/>
         <v>6290</v>
       </c>
       <c r="I11" s="11">
-        <f>IF(F11=0,0,H11/F11)</f>
+        <f t="shared" si="1"/>
         <v>0.29669811320754719</v>
       </c>
     </row>
@@ -2564,11 +2561,11 @@
         <v>72220</v>
       </c>
       <c r="H12" s="16">
-        <f>G12-F12</f>
+        <f t="shared" si="0"/>
         <v>16480</v>
       </c>
       <c r="I12" s="11">
-        <f>IF(F12=0,0,H12/F12)</f>
+        <f t="shared" si="1"/>
         <v>0.29565841406530319</v>
       </c>
     </row>
@@ -2595,11 +2592,11 @@
         <v>11400</v>
       </c>
       <c r="H13" s="6">
-        <f>G13-F13</f>
+        <f t="shared" si="0"/>
         <v>2600</v>
       </c>
       <c r="I13" s="11">
-        <f>IF(F13=0,0,H13/F13)</f>
+        <f t="shared" si="1"/>
         <v>0.29545454545454547</v>
       </c>
     </row>
@@ -2626,11 +2623,11 @@
         <v>765470</v>
       </c>
       <c r="H14" s="16">
-        <f>G14-F14</f>
+        <f t="shared" si="0"/>
         <v>174510</v>
       </c>
       <c r="I14" s="11">
-        <f>IF(F14=0,0,H14/F14)</f>
+        <f t="shared" si="1"/>
         <v>0.29529917422498986</v>
       </c>
     </row>
@@ -2657,11 +2654,11 @@
         <v>21630</v>
       </c>
       <c r="H15" s="6">
-        <f>G15-F15</f>
+        <f t="shared" si="0"/>
         <v>4930</v>
       </c>
       <c r="I15" s="11">
-        <f>IF(F15=0,0,H15/F15)</f>
+        <f t="shared" si="1"/>
         <v>0.29520958083832333</v>
       </c>
     </row>
@@ -2688,11 +2685,11 @@
         <v>40840</v>
       </c>
       <c r="H16" s="6">
-        <f>G16-F16</f>
+        <f t="shared" si="0"/>
         <v>9300</v>
       </c>
       <c r="I16" s="11">
-        <f>IF(F16=0,0,H16/F16)</f>
+        <f t="shared" si="1"/>
         <v>0.29486366518706403</v>
       </c>
     </row>
@@ -2719,11 +2716,11 @@
         <v>14010</v>
       </c>
       <c r="H17" s="6">
-        <f>G17-F17</f>
+        <f t="shared" si="0"/>
         <v>3190</v>
       </c>
       <c r="I17" s="11">
-        <f>IF(F17=0,0,H17/F17)</f>
+        <f t="shared" si="1"/>
         <v>0.29482439926062848</v>
       </c>
     </row>
@@ -2750,11 +2747,11 @@
         <v>29560</v>
       </c>
       <c r="H18" s="6">
-        <f>G18-F18</f>
+        <f t="shared" si="0"/>
         <v>6720</v>
       </c>
       <c r="I18" s="11">
-        <f>IF(F18=0,0,H18/F18)</f>
+        <f t="shared" si="1"/>
         <v>0.29422066549912435</v>
       </c>
     </row>
@@ -2781,11 +2778,11 @@
         <v>109950</v>
       </c>
       <c r="H19" s="16">
-        <f>G19-F19</f>
+        <f t="shared" si="0"/>
         <v>24910</v>
       </c>
       <c r="I19" s="11">
-        <f>IF(F19=0,0,H19/F19)</f>
+        <f t="shared" si="1"/>
         <v>0.29292097836312325</v>
       </c>
     </row>
@@ -2812,11 +2809,11 @@
         <v>17181</v>
       </c>
       <c r="H20" s="6">
-        <f>G20-F20</f>
+        <f t="shared" si="0"/>
         <v>2469</v>
       </c>
       <c r="I20" s="11">
-        <f>IF(F20=0,0,H20/F20)</f>
+        <f t="shared" si="1"/>
         <v>0.16782218597063622</v>
       </c>
     </row>
@@ -2843,11 +2840,11 @@
         <v>574340</v>
       </c>
       <c r="H21" s="16">
-        <f>G21-F21</f>
+        <f t="shared" si="0"/>
         <v>38470</v>
       </c>
       <c r="I21" s="7">
-        <f>IF(F21=0,0,H21/F21)</f>
+        <f t="shared" si="1"/>
         <v>7.1789799764868351E-2</v>
       </c>
     </row>
@@ -2874,11 +2871,11 @@
         <v>7297</v>
       </c>
       <c r="H22" s="6">
-        <f>G22-F22</f>
+        <f t="shared" si="0"/>
         <v>356</v>
       </c>
       <c r="I22" s="7">
-        <f>IF(F22=0,0,H22/F22)</f>
+        <f t="shared" si="1"/>
         <v>5.1289439562022761E-2</v>
       </c>
     </row>
@@ -2905,11 +2902,11 @@
         <v>4176</v>
       </c>
       <c r="H23" s="6">
-        <f>G23-F23</f>
+        <f t="shared" si="0"/>
         <v>193</v>
       </c>
       <c r="I23" s="7">
-        <f>IF(F23=0,0,H23/F23)</f>
+        <f t="shared" si="1"/>
         <v>4.8455937735375348E-2</v>
       </c>
     </row>
@@ -2936,11 +2933,11 @@
         <v>71</v>
       </c>
       <c r="H24" s="6">
-        <f>G24-F24</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="I24" s="7">
-        <f>IF(F24=0,0,H24/F24)</f>
+        <f t="shared" si="1"/>
         <v>4.4117647058823532E-2</v>
       </c>
     </row>
@@ -2967,11 +2964,11 @@
         <v>306</v>
       </c>
       <c r="H25" s="6">
-        <f>G25-F25</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="I25" s="7">
-        <f>IF(F25=0,0,H25/F25)</f>
+        <f t="shared" si="1"/>
         <v>4.0816326530612242E-2</v>
       </c>
     </row>
@@ -2998,11 +2995,11 @@
         <v>643</v>
       </c>
       <c r="H26" s="6">
-        <f>G26-F26</f>
+        <f t="shared" si="0"/>
         <v>25</v>
       </c>
       <c r="I26" s="7">
-        <f>IF(F26=0,0,H26/F26)</f>
+        <f t="shared" si="1"/>
         <v>4.0453074433656956E-2</v>
       </c>
     </row>
@@ -3029,11 +3026,11 @@
         <v>336</v>
       </c>
       <c r="H27" s="6">
-        <f>G27-F27</f>
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="I27" s="7">
-        <f>IF(F27=0,0,H27/F27)</f>
+        <f t="shared" si="1"/>
         <v>4.0247678018575851E-2</v>
       </c>
     </row>
@@ -3060,11 +3057,11 @@
         <v>51118</v>
       </c>
       <c r="H28" s="6">
-        <f>G28-F28</f>
+        <f t="shared" si="0"/>
         <v>1968</v>
       </c>
       <c r="I28" s="7">
-        <f>IF(F28=0,0,H28/F28)</f>
+        <f t="shared" si="1"/>
         <v>4.0040691759918617E-2</v>
       </c>
     </row>
@@ -3091,11 +3088,11 @@
         <v>79</v>
       </c>
       <c r="H29" s="6">
-        <f>G29-F29</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="I29" s="7">
-        <f>IF(F29=0,0,H29/F29)</f>
+        <f t="shared" si="1"/>
         <v>3.9473684210526314E-2</v>
       </c>
     </row>
@@ -3122,11 +3119,11 @@
         <v>609</v>
       </c>
       <c r="H30" s="6">
-        <f>G30-F30</f>
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="I30" s="7">
-        <f>IF(F30=0,0,H30/F30)</f>
+        <f t="shared" si="1"/>
         <v>3.9249146757679182E-2</v>
       </c>
     </row>
@@ -3153,11 +3150,11 @@
         <v>106</v>
       </c>
       <c r="H31" s="6">
-        <f>G31-F31</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="I31" s="7">
-        <f>IF(F31=0,0,H31/F31)</f>
+        <f t="shared" si="1"/>
         <v>3.9215686274509803E-2</v>
       </c>
     </row>
@@ -3184,11 +3181,11 @@
         <v>1488</v>
       </c>
       <c r="H32" s="6">
-        <f>G32-F32</f>
+        <f t="shared" si="0"/>
         <v>56</v>
       </c>
       <c r="I32" s="7">
-        <f>IF(F32=0,0,H32/F32)</f>
+        <f t="shared" si="1"/>
         <v>3.9106145251396648E-2</v>
       </c>
     </row>
@@ -3215,11 +3212,11 @@
         <v>1329</v>
       </c>
       <c r="H33" s="6">
-        <f>G33-F33</f>
+        <f t="shared" si="0"/>
         <v>50</v>
       </c>
       <c r="I33" s="7">
-        <f>IF(F33=0,0,H33/F33)</f>
+        <f t="shared" si="1"/>
         <v>3.9093041438623924E-2</v>
       </c>
     </row>
@@ -3246,11 +3243,11 @@
         <v>586</v>
       </c>
       <c r="H34" s="6">
-        <f>G34-F34</f>
+        <f t="shared" ref="H34:H65" si="2">G34-F34</f>
         <v>22</v>
       </c>
       <c r="I34" s="7">
-        <f>IF(F34=0,0,H34/F34)</f>
+        <f t="shared" ref="I34:I65" si="3">IF(F34=0,0,H34/F34)</f>
         <v>3.9007092198581561E-2</v>
       </c>
     </row>
@@ -3277,11 +3274,11 @@
         <v>4401</v>
       </c>
       <c r="H35" s="6">
-        <f>G35-F35</f>
+        <f t="shared" si="2"/>
         <v>165</v>
       </c>
       <c r="I35" s="7">
-        <f>IF(F35=0,0,H35/F35)</f>
+        <f t="shared" si="3"/>
         <v>3.8951841359773372E-2</v>
       </c>
     </row>
@@ -3308,11 +3305,11 @@
         <v>1894</v>
       </c>
       <c r="H36" s="6">
-        <f>G36-F36</f>
+        <f t="shared" si="2"/>
         <v>71</v>
       </c>
       <c r="I36" s="7">
-        <f>IF(F36=0,0,H36/F36)</f>
+        <f t="shared" si="3"/>
         <v>3.8946791003839826E-2</v>
       </c>
     </row>
@@ -3339,11 +3336,11 @@
         <v>1522</v>
       </c>
       <c r="H37" s="6">
-        <f>G37-F37</f>
+        <f t="shared" si="2"/>
         <v>57</v>
       </c>
       <c r="I37" s="7">
-        <f>IF(F37=0,0,H37/F37)</f>
+        <f t="shared" si="3"/>
         <v>3.8907849829351533E-2</v>
       </c>
     </row>
@@ -3370,11 +3367,11 @@
         <v>1309</v>
       </c>
       <c r="H38" s="6">
-        <f>G38-F38</f>
+        <f t="shared" si="2"/>
         <v>49</v>
       </c>
       <c r="I38" s="7">
-        <f>IF(F38=0,0,H38/F38)</f>
+        <f t="shared" si="3"/>
         <v>3.888888888888889E-2</v>
       </c>
     </row>
@@ -3401,11 +3398,11 @@
         <v>5692</v>
       </c>
       <c r="H39" s="6">
-        <f>G39-F39</f>
+        <f t="shared" si="2"/>
         <v>213</v>
       </c>
       <c r="I39" s="7">
-        <f>IF(F39=0,0,H39/F39)</f>
+        <f t="shared" si="3"/>
         <v>3.8875707245847782E-2</v>
       </c>
     </row>
@@ -3432,11 +3429,11 @@
         <v>990</v>
       </c>
       <c r="H40" s="6">
-        <f>G40-F40</f>
+        <f t="shared" si="2"/>
         <v>37</v>
       </c>
       <c r="I40" s="7">
-        <f>IF(F40=0,0,H40/F40)</f>
+        <f t="shared" si="3"/>
         <v>3.8824763903462747E-2</v>
       </c>
     </row>
@@ -3463,11 +3460,11 @@
         <v>5436</v>
       </c>
       <c r="H41" s="6">
-        <f>G41-F41</f>
+        <f t="shared" si="2"/>
         <v>203</v>
       </c>
       <c r="I41" s="7">
-        <f>IF(F41=0,0,H41/F41)</f>
+        <f t="shared" si="3"/>
         <v>3.8792279763042233E-2</v>
       </c>
     </row>
@@ -3494,11 +3491,11 @@
         <v>3536</v>
       </c>
       <c r="H42" s="6">
-        <f>G42-F42</f>
+        <f t="shared" si="2"/>
         <v>132</v>
       </c>
       <c r="I42" s="7">
-        <f>IF(F42=0,0,H42/F42)</f>
+        <f t="shared" si="3"/>
         <v>3.8777908343125736E-2</v>
       </c>
     </row>
@@ -3525,11 +3522,11 @@
         <v>134</v>
       </c>
       <c r="H43" s="6">
-        <f>G43-F43</f>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
       <c r="I43" s="7">
-        <f>IF(F43=0,0,H43/F43)</f>
+        <f t="shared" si="3"/>
         <v>3.875968992248062E-2</v>
       </c>
     </row>
@@ -3556,11 +3553,11 @@
         <v>3404</v>
       </c>
       <c r="H44" s="6">
-        <f>G44-F44</f>
+        <f t="shared" si="2"/>
         <v>127</v>
       </c>
       <c r="I44" s="7">
-        <f>IF(F44=0,0,H44/F44)</f>
+        <f t="shared" si="3"/>
         <v>3.8754958803783948E-2</v>
       </c>
     </row>
@@ -3587,11 +3584,11 @@
         <v>322</v>
       </c>
       <c r="H45" s="6">
-        <f>G45-F45</f>
+        <f t="shared" si="2"/>
         <v>12</v>
       </c>
       <c r="I45" s="7">
-        <f>IF(F45=0,0,H45/F45)</f>
+        <f t="shared" si="3"/>
         <v>3.870967741935484E-2</v>
       </c>
     </row>
@@ -3618,11 +3615,11 @@
         <v>1906</v>
       </c>
       <c r="H46" s="6">
-        <f>G46-F46</f>
+        <f t="shared" si="2"/>
         <v>71</v>
       </c>
       <c r="I46" s="7">
-        <f>IF(F46=0,0,H46/F46)</f>
+        <f t="shared" si="3"/>
         <v>3.8692098092643054E-2</v>
       </c>
     </row>
@@ -3649,11 +3646,11 @@
         <v>215</v>
       </c>
       <c r="H47" s="6">
-        <f>G47-F47</f>
+        <f t="shared" si="2"/>
         <v>8</v>
       </c>
       <c r="I47" s="7">
-        <f>IF(F47=0,0,H47/F47)</f>
+        <f t="shared" si="3"/>
         <v>3.864734299516908E-2</v>
       </c>
     </row>
@@ -3680,11 +3677,11 @@
         <v>1345</v>
       </c>
       <c r="H48" s="6">
-        <f>G48-F48</f>
+        <f t="shared" si="2"/>
         <v>50</v>
       </c>
       <c r="I48" s="7">
-        <f>IF(F48=0,0,H48/F48)</f>
+        <f t="shared" si="3"/>
         <v>3.8610038610038609E-2</v>
       </c>
     </row>
@@ -3711,11 +3708,11 @@
         <v>1349</v>
       </c>
       <c r="H49" s="6">
-        <f>G49-F49</f>
+        <f t="shared" si="2"/>
         <v>50</v>
       </c>
       <c r="I49" s="7">
-        <f>IF(F49=0,0,H49/F49)</f>
+        <f t="shared" si="3"/>
         <v>3.8491147036181679E-2</v>
       </c>
     </row>
@@ -3742,11 +3739,11 @@
         <v>324</v>
       </c>
       <c r="H50" s="6">
-        <f>G50-F50</f>
+        <f t="shared" si="2"/>
         <v>12</v>
       </c>
       <c r="I50" s="7">
-        <f>IF(F50=0,0,H50/F50)</f>
+        <f t="shared" si="3"/>
         <v>3.8461538461538464E-2</v>
       </c>
     </row>
@@ -3773,11 +3770,11 @@
         <v>517</v>
       </c>
       <c r="H51" s="6">
-        <f>G51-F51</f>
+        <f t="shared" si="2"/>
         <v>19</v>
       </c>
       <c r="I51" s="7">
-        <f>IF(F51=0,0,H51/F51)</f>
+        <f t="shared" si="3"/>
         <v>3.8152610441767071E-2</v>
       </c>
     </row>
@@ -3804,11 +3801,11 @@
         <v>273</v>
       </c>
       <c r="H52" s="6">
-        <f>G52-F52</f>
+        <f t="shared" si="2"/>
         <v>10</v>
       </c>
       <c r="I52" s="7">
-        <f>IF(F52=0,0,H52/F52)</f>
+        <f t="shared" si="3"/>
         <v>3.8022813688212927E-2</v>
       </c>
     </row>
@@ -3835,11 +3832,11 @@
         <v>362.44</v>
       </c>
       <c r="H53" s="6">
-        <f>G53-F53</f>
+        <f t="shared" si="2"/>
         <v>13</v>
       </c>
       <c r="I53" s="7">
-        <f>IF(F53=0,0,H53/F53)</f>
+        <f t="shared" si="3"/>
         <v>3.7202380952380952E-2</v>
       </c>
     </row>
@@ -3866,11 +3863,11 @@
         <v>60</v>
       </c>
       <c r="H54" s="6">
-        <f>G54-F54</f>
+        <f t="shared" si="2"/>
         <v>2</v>
       </c>
       <c r="I54" s="7">
-        <f>IF(F54=0,0,H54/F54)</f>
+        <f t="shared" si="3"/>
         <v>3.4482758620689655E-2</v>
       </c>
     </row>
@@ -3897,11 +3894,11 @@
         <v>42912.3</v>
       </c>
       <c r="H55" s="6">
-        <f>G55-F55</f>
+        <f t="shared" si="2"/>
         <v>1411</v>
       </c>
       <c r="I55" s="7">
-        <f>IF(F55=0,0,H55/F55)</f>
+        <f t="shared" si="3"/>
         <v>3.3998934973121321E-2</v>
       </c>
     </row>
@@ -3928,11 +3925,11 @@
         <v>329875</v>
       </c>
       <c r="H56" s="16">
-        <f>G56-F56</f>
+        <f t="shared" si="2"/>
         <v>10700</v>
       </c>
       <c r="I56" s="7">
-        <f>IF(F56=0,0,H56/F56)</f>
+        <f t="shared" si="3"/>
         <v>3.3523928879141539E-2</v>
       </c>
     </row>
@@ -3959,11 +3956,11 @@
         <v>111074</v>
       </c>
       <c r="H57" s="6">
-        <f>G57-F57</f>
+        <f t="shared" si="2"/>
         <v>3000</v>
       </c>
       <c r="I57" s="7">
-        <f>IF(F57=0,0,H57/F57)</f>
+        <f t="shared" si="3"/>
         <v>2.7758757888113699E-2</v>
       </c>
     </row>
@@ -3990,11 +3987,11 @@
         <v>6654</v>
       </c>
       <c r="H58" s="6">
-        <f>G58-F58</f>
+        <f t="shared" si="2"/>
         <v>177</v>
       </c>
       <c r="I58" s="7">
-        <f>IF(F58=0,0,H58/F58)</f>
+        <f t="shared" si="3"/>
         <v>2.7327466419638721E-2</v>
       </c>
     </row>
@@ -4021,11 +4018,11 @@
         <v>385870.59499999997</v>
       </c>
       <c r="H59" s="16">
-        <f>G59-F59</f>
+        <f t="shared" si="2"/>
         <v>10134.030999999959</v>
       </c>
       <c r="I59" s="7">
-        <f>IF(F59=0,0,H59/F59)</f>
+        <f t="shared" si="3"/>
         <v>2.6971106809823168E-2</v>
       </c>
     </row>
@@ -4052,11 +4049,11 @@
         <v>76698</v>
       </c>
       <c r="H60" s="6">
-        <f>G60-F60</f>
+        <f t="shared" si="2"/>
         <v>1894</v>
       </c>
       <c r="I60" s="7">
-        <f>IF(F60=0,0,H60/F60)</f>
+        <f t="shared" si="3"/>
         <v>2.5319501630928828E-2</v>
       </c>
     </row>
@@ -4083,11 +4080,11 @@
         <v>99705</v>
       </c>
       <c r="H61" s="6">
-        <f>G61-F61</f>
+        <f t="shared" si="2"/>
         <v>2103</v>
       </c>
       <c r="I61" s="7">
-        <f>IF(F61=0,0,H61/F61)</f>
+        <f t="shared" si="3"/>
         <v>2.1546689617016043E-2</v>
       </c>
     </row>
@@ -4114,11 +4111,11 @@
         <v>183047</v>
       </c>
       <c r="H62" s="6">
-        <f>G62-F62</f>
+        <f t="shared" si="2"/>
         <v>3651</v>
       </c>
       <c r="I62" s="7">
-        <f>IF(F62=0,0,H62/F62)</f>
+        <f t="shared" si="3"/>
         <v>2.0351624339450154E-2</v>
       </c>
     </row>
@@ -4145,11 +4142,11 @@
         <v>49497</v>
       </c>
       <c r="H63" s="6">
-        <f>G63-F63</f>
+        <f t="shared" si="2"/>
         <v>950</v>
       </c>
       <c r="I63" s="7">
-        <f>IF(F63=0,0,H63/F63)</f>
+        <f t="shared" si="3"/>
         <v>1.9568665417018561E-2</v>
       </c>
     </row>
@@ -4176,11 +4173,11 @@
         <v>5267</v>
       </c>
       <c r="H64" s="6">
-        <f>G64-F64</f>
+        <f t="shared" si="2"/>
         <v>93</v>
       </c>
       <c r="I64" s="7">
-        <f>IF(F64=0,0,H64/F64)</f>
+        <f t="shared" si="3"/>
         <v>1.7974487823734054E-2</v>
       </c>
     </row>
@@ -4207,11 +4204,11 @@
         <v>15334</v>
       </c>
       <c r="H65" s="6">
-        <f>G65-F65</f>
+        <f t="shared" si="2"/>
         <v>232</v>
       </c>
       <c r="I65" s="7">
-        <f>IF(F65=0,0,H65/F65)</f>
+        <f t="shared" si="3"/>
         <v>1.5362203681631572E-2</v>
       </c>
     </row>
@@ -4238,11 +4235,11 @@
         <v>26580</v>
       </c>
       <c r="H66" s="6">
-        <f>G66-F66</f>
+        <f t="shared" ref="H66:H97" si="4">G66-F66</f>
         <v>350</v>
       </c>
       <c r="I66" s="7">
-        <f>IF(F66=0,0,H66/F66)</f>
+        <f t="shared" ref="I66:I97" si="5">IF(F66=0,0,H66/F66)</f>
         <v>1.3343499809378575E-2</v>
       </c>
     </row>
@@ -4269,11 +4266,11 @@
         <v>19973</v>
       </c>
       <c r="H67" s="6">
-        <f>G67-F67</f>
+        <f t="shared" si="4"/>
         <v>263</v>
       </c>
       <c r="I67" s="7">
-        <f>IF(F67=0,0,H67/F67)</f>
+        <f t="shared" si="5"/>
         <v>1.3343480466768138E-2</v>
       </c>
     </row>
@@ -4300,11 +4297,11 @@
         <v>30342</v>
       </c>
       <c r="H68" s="6">
-        <f>G68-F68</f>
+        <f t="shared" si="4"/>
         <v>399</v>
       </c>
       <c r="I68" s="7">
-        <f>IF(F68=0,0,H68/F68)</f>
+        <f t="shared" si="5"/>
         <v>1.3325318104398357E-2</v>
       </c>
     </row>
@@ -4331,11 +4328,11 @@
         <v>22900</v>
       </c>
       <c r="H69" s="6">
-        <f>G69-F69</f>
+        <f t="shared" si="4"/>
         <v>291</v>
       </c>
       <c r="I69" s="7">
-        <f>IF(F69=0,0,H69/F69)</f>
+        <f t="shared" si="5"/>
         <v>1.2870980582953691E-2</v>
       </c>
     </row>
@@ -4362,11 +4359,11 @@
         <v>25990</v>
       </c>
       <c r="H70" s="6">
-        <f>G70-F70</f>
+        <f t="shared" si="4"/>
         <v>313</v>
       </c>
       <c r="I70" s="7">
-        <f>IF(F70=0,0,H70/F70)</f>
+        <f t="shared" si="5"/>
         <v>1.2189897573704093E-2</v>
       </c>
     </row>
@@ -4393,11 +4390,11 @@
         <v>2195</v>
       </c>
       <c r="H71" s="6">
-        <f>G71-F71</f>
+        <f t="shared" si="4"/>
         <v>23</v>
       </c>
       <c r="I71" s="7">
-        <f>IF(F71=0,0,H71/F71)</f>
+        <f t="shared" si="5"/>
         <v>1.0589318600368325E-2</v>
       </c>
     </row>
@@ -4424,11 +4421,11 @@
         <v>589</v>
       </c>
       <c r="H72" s="6">
-        <f>G72-F72</f>
+        <f t="shared" si="4"/>
         <v>6</v>
       </c>
       <c r="I72" s="7">
-        <f>IF(F72=0,0,H72/F72)</f>
+        <f t="shared" si="5"/>
         <v>1.0291595197255575E-2</v>
       </c>
     </row>
@@ -4455,11 +4452,11 @@
         <v>1277</v>
       </c>
       <c r="H73" s="6">
-        <f>G73-F73</f>
+        <f t="shared" si="4"/>
         <v>13</v>
       </c>
       <c r="I73" s="7">
-        <f>IF(F73=0,0,H73/F73)</f>
+        <f t="shared" si="5"/>
         <v>1.0284810126582278E-2</v>
       </c>
     </row>
@@ -4486,11 +4483,11 @@
         <v>2658</v>
       </c>
       <c r="H74" s="6">
-        <f>G74-F74</f>
+        <f t="shared" si="4"/>
         <v>27</v>
       </c>
       <c r="I74" s="7">
-        <f>IF(F74=0,0,H74/F74)</f>
+        <f t="shared" si="5"/>
         <v>1.0262257696693273E-2</v>
       </c>
     </row>
@@ -4517,11 +4514,11 @@
         <v>4251</v>
       </c>
       <c r="H75" s="6">
-        <f>G75-F75</f>
+        <f t="shared" si="4"/>
         <v>43</v>
       </c>
       <c r="I75" s="7">
-        <f>IF(F75=0,0,H75/F75)</f>
+        <f t="shared" si="5"/>
         <v>1.0218631178707225E-2</v>
       </c>
     </row>
@@ -4548,11 +4545,11 @@
         <v>1286</v>
       </c>
       <c r="H76" s="6">
-        <f>G76-F76</f>
+        <f t="shared" si="4"/>
         <v>13</v>
       </c>
       <c r="I76" s="7">
-        <f>IF(F76=0,0,H76/F76)</f>
+        <f t="shared" si="5"/>
         <v>1.0212097407698351E-2</v>
       </c>
     </row>
@@ -4579,11 +4576,11 @@
         <v>7974</v>
       </c>
       <c r="H77" s="6">
-        <f>G77-F77</f>
+        <f t="shared" si="4"/>
         <v>80</v>
       </c>
       <c r="I77" s="7">
-        <f>IF(F77=0,0,H77/F77)</f>
+        <f t="shared" si="5"/>
         <v>1.0134279199391943E-2</v>
       </c>
     </row>
@@ -4610,11 +4607,11 @@
         <v>1798</v>
       </c>
       <c r="H78" s="6">
-        <f>G78-F78</f>
+        <f t="shared" si="4"/>
         <v>18</v>
       </c>
       <c r="I78" s="7">
-        <f>IF(F78=0,0,H78/F78)</f>
+        <f t="shared" si="5"/>
         <v>1.0112359550561797E-2</v>
       </c>
     </row>
@@ -4641,11 +4638,11 @@
         <v>29703.937000000002</v>
       </c>
       <c r="H79" s="6">
-        <f>G79-F79</f>
+        <f t="shared" si="4"/>
         <v>297</v>
       </c>
       <c r="I79" s="7">
-        <f>IF(F79=0,0,H79/F79)</f>
+        <f t="shared" si="5"/>
         <v>1.0099657778027E-2</v>
       </c>
     </row>
@@ -4672,11 +4669,11 @@
         <v>44309</v>
       </c>
       <c r="H80" s="6">
-        <f>G80-F80</f>
+        <f t="shared" si="4"/>
         <v>443</v>
       </c>
       <c r="I80" s="7">
-        <f>IF(F80=0,0,H80/F80)</f>
+        <f t="shared" si="5"/>
         <v>1.009893767382483E-2</v>
       </c>
     </row>
@@ -4703,11 +4700,11 @@
         <v>18405.45</v>
       </c>
       <c r="H81" s="6">
-        <f>G81-F81</f>
+        <f t="shared" si="4"/>
         <v>184</v>
       </c>
       <c r="I81" s="7">
-        <f>IF(F81=0,0,H81/F81)</f>
+        <f t="shared" si="5"/>
         <v>1.0097988908676312E-2</v>
       </c>
     </row>
@@ -4734,11 +4731,11 @@
         <v>22312</v>
       </c>
       <c r="H82" s="6">
-        <f>G82-F82</f>
+        <f t="shared" si="4"/>
         <v>223</v>
       </c>
       <c r="I82" s="7">
-        <f>IF(F82=0,0,H82/F82)</f>
+        <f t="shared" si="5"/>
         <v>1.0095522658336728E-2</v>
       </c>
     </row>
@@ -4765,11 +4762,11 @@
         <v>6111</v>
       </c>
       <c r="H83" s="6">
-        <f>G83-F83</f>
+        <f t="shared" si="4"/>
         <v>61</v>
       </c>
       <c r="I83" s="7">
-        <f>IF(F83=0,0,H83/F83)</f>
+        <f t="shared" si="5"/>
         <v>1.0082644628099173E-2</v>
       </c>
     </row>
@@ -4796,11 +4793,11 @@
         <v>2204</v>
       </c>
       <c r="H84" s="6">
-        <f>G84-F84</f>
+        <f t="shared" si="4"/>
         <v>22</v>
       </c>
       <c r="I84" s="7">
-        <f>IF(F84=0,0,H84/F84)</f>
+        <f t="shared" si="5"/>
         <v>1.0082493125572869E-2</v>
       </c>
     </row>
@@ -4827,11 +4824,11 @@
         <v>10633</v>
       </c>
       <c r="H85" s="6">
-        <f>G85-F85</f>
+        <f t="shared" si="4"/>
         <v>106</v>
       </c>
       <c r="I85" s="7">
-        <f>IF(F85=0,0,H85/F85)</f>
+        <f t="shared" si="5"/>
         <v>1.0069345492542984E-2</v>
       </c>
     </row>
@@ -4858,11 +4855,11 @@
         <v>9530</v>
       </c>
       <c r="H86" s="6">
-        <f>G86-F86</f>
+        <f t="shared" si="4"/>
         <v>95</v>
       </c>
       <c r="I86" s="7">
-        <f>IF(F86=0,0,H86/F86)</f>
+        <f t="shared" si="5"/>
         <v>1.0068892421833599E-2</v>
       </c>
     </row>
@@ -4889,11 +4886,11 @@
         <v>5720</v>
       </c>
       <c r="H87" s="6">
-        <f>G87-F87</f>
+        <f t="shared" si="4"/>
         <v>57</v>
       </c>
       <c r="I87" s="7">
-        <f>IF(F87=0,0,H87/F87)</f>
+        <f t="shared" si="5"/>
         <v>1.0065336394137384E-2</v>
       </c>
     </row>
@@ -4920,11 +4917,11 @@
         <v>5725</v>
       </c>
       <c r="H88" s="6">
-        <f>G88-F88</f>
+        <f t="shared" si="4"/>
         <v>57</v>
       </c>
       <c r="I88" s="7">
-        <f>IF(F88=0,0,H88/F88)</f>
+        <f t="shared" si="5"/>
         <v>1.0056457304163727E-2</v>
       </c>
     </row>
@@ -4951,11 +4948,11 @@
         <v>1123300</v>
       </c>
       <c r="H89" s="16">
-        <f>G89-F89</f>
+        <f t="shared" si="4"/>
         <v>10970</v>
       </c>
       <c r="I89" s="7">
-        <f>IF(F89=0,0,H89/F89)</f>
+        <f t="shared" si="5"/>
         <v>9.8621811872375998E-3</v>
       </c>
     </row>
@@ -4982,11 +4979,11 @@
         <v>4011</v>
       </c>
       <c r="H90" s="6">
-        <f>G90-F90</f>
+        <f t="shared" si="4"/>
         <v>39</v>
       </c>
       <c r="I90" s="7">
-        <f>IF(F90=0,0,H90/F90)</f>
+        <f t="shared" si="5"/>
         <v>9.8187311178247732E-3</v>
       </c>
     </row>
@@ -5013,11 +5010,11 @@
         <v>2366.13</v>
       </c>
       <c r="H91" s="6">
-        <f>G91-F91</f>
+        <f t="shared" si="4"/>
         <v>23</v>
       </c>
       <c r="I91" s="7">
-        <f>IF(F91=0,0,H91/F91)</f>
+        <f t="shared" si="5"/>
         <v>9.8159299740091244E-3</v>
       </c>
     </row>
@@ -5044,11 +5041,11 @@
         <v>5457</v>
       </c>
       <c r="H92" s="6">
-        <f>G92-F92</f>
+        <f t="shared" si="4"/>
         <v>53</v>
       </c>
       <c r="I92" s="7">
-        <f>IF(F92=0,0,H92/F92)</f>
+        <f t="shared" si="5"/>
         <v>9.8075499629903772E-3</v>
       </c>
     </row>
@@ -5075,11 +5072,11 @@
         <v>16211</v>
       </c>
       <c r="H93" s="6">
-        <f>G93-F93</f>
+        <f t="shared" si="4"/>
         <v>155</v>
       </c>
       <c r="I93" s="7">
-        <f>IF(F93=0,0,H93/F93)</f>
+        <f t="shared" si="5"/>
         <v>9.653712007972097E-3</v>
       </c>
     </row>
@@ -5106,11 +5103,11 @@
         <v>945</v>
       </c>
       <c r="H94" s="6">
-        <f>G94-F94</f>
+        <f t="shared" si="4"/>
         <v>9</v>
       </c>
       <c r="I94" s="7">
-        <f>IF(F94=0,0,H94/F94)</f>
+        <f t="shared" si="5"/>
         <v>9.6153846153846159E-3</v>
       </c>
     </row>
@@ -5137,11 +5134,11 @@
         <v>985</v>
       </c>
       <c r="H95" s="6">
-        <f>G95-F95</f>
+        <f t="shared" si="4"/>
         <v>9</v>
       </c>
       <c r="I95" s="7">
-        <f>IF(F95=0,0,H95/F95)</f>
+        <f t="shared" si="5"/>
         <v>9.2213114754098359E-3</v>
       </c>
     </row>
@@ -5168,11 +5165,11 @@
         <v>13595.65</v>
       </c>
       <c r="H96" s="6">
-        <f>G96-F96</f>
+        <f t="shared" si="4"/>
         <v>116</v>
       </c>
       <c r="I96" s="7">
-        <f>IF(F96=0,0,H96/F96)</f>
+        <f t="shared" si="5"/>
         <v>8.6055646845429965E-3</v>
       </c>
     </row>
@@ -5199,11 +5196,11 @@
         <v>713</v>
       </c>
       <c r="H97" s="6">
-        <f>G97-F97</f>
+        <f t="shared" si="4"/>
         <v>6</v>
       </c>
       <c r="I97" s="7">
-        <f>IF(F97=0,0,H97/F97)</f>
+        <f t="shared" si="5"/>
         <v>8.4865629420084864E-3</v>
       </c>
     </row>
@@ -5230,11 +5227,11 @@
         <v>1628</v>
       </c>
       <c r="H98" s="6">
-        <f>G98-F98</f>
+        <f t="shared" ref="H98:H129" si="6">G98-F98</f>
         <v>13</v>
       </c>
       <c r="I98" s="7">
-        <f>IF(F98=0,0,H98/F98)</f>
+        <f t="shared" ref="I98:I129" si="7">IF(F98=0,0,H98/F98)</f>
         <v>8.0495356037151699E-3</v>
       </c>
     </row>
@@ -5261,11 +5258,11 @@
         <v>547174.81499999994</v>
       </c>
       <c r="H99" s="6">
-        <f>G99-F99</f>
+        <f t="shared" si="6"/>
         <v>491.3179999999702</v>
       </c>
       <c r="I99" s="7">
-        <f>IF(F99=0,0,H99/F99)</f>
+        <f t="shared" si="7"/>
         <v>8.9872476980948671E-4</v>
       </c>
     </row>
@@ -5292,11 +5289,11 @@
         <v>10605.808000000001</v>
       </c>
       <c r="H100" s="6">
-        <f>G100-F100</f>
+        <f t="shared" si="6"/>
         <v>3.9240000000008877</v>
       </c>
       <c r="I100" s="7">
-        <f>IF(F100=0,0,H100/F100)</f>
+        <f t="shared" si="7"/>
         <v>3.7012289513834405E-4</v>
       </c>
     </row>
@@ -5323,11 +5320,11 @@
         <v>25718.210999999999</v>
       </c>
       <c r="H101" s="6">
-        <f>G101-F101</f>
+        <f t="shared" si="6"/>
         <v>9.4140000000006694</v>
       </c>
       <c r="I101" s="7">
-        <f>IF(F101=0,0,H101/F101)</f>
+        <f t="shared" si="7"/>
         <v>3.6617816072843354E-4</v>
       </c>
     </row>
@@ -5354,11 +5351,11 @@
         <v>31865.093000000001</v>
       </c>
       <c r="H102" s="6">
-        <f>G102-F102</f>
+        <f t="shared" si="6"/>
         <v>11.619000000002416</v>
       </c>
       <c r="I102" s="7">
-        <f>IF(F102=0,0,H102/F102)</f>
+        <f t="shared" si="7"/>
         <v>3.6476398147349378E-4</v>
       </c>
     </row>
@@ -5385,11 +5382,11 @@
         <v>19489.734</v>
       </c>
       <c r="H103" s="6">
-        <f>G103-F103</f>
+        <f t="shared" si="6"/>
         <v>6.9570000000021537</v>
       </c>
       <c r="I103" s="7">
-        <f>IF(F103=0,0,H103/F103)</f>
+        <f t="shared" si="7"/>
         <v>3.570846188919657E-4</v>
       </c>
     </row>
@@ -5416,11 +5413,11 @@
         <v>144035.94</v>
       </c>
       <c r="H104" s="6">
-        <f>G104-F104</f>
+        <f t="shared" si="6"/>
         <v>51.358000000007451</v>
       </c>
       <c r="I104" s="7">
-        <f>IF(F104=0,0,H104/F104)</f>
+        <f t="shared" si="7"/>
         <v>3.5669096848166319E-4</v>
       </c>
     </row>
@@ -5447,11 +5444,11 @@
         <v>102480.54399999999</v>
       </c>
       <c r="H105" s="6">
-        <f>G105-F105</f>
+        <f t="shared" si="6"/>
         <v>36.273999999990338</v>
       </c>
       <c r="I105" s="7">
-        <f>IF(F105=0,0,H105/F105)</f>
+        <f t="shared" si="7"/>
         <v>3.5408520164173491E-4</v>
       </c>
     </row>
@@ -5478,11 +5475,11 @@
         <v>106390.065</v>
       </c>
       <c r="H106" s="6">
-        <f>G106-F106</f>
+        <f t="shared" si="6"/>
         <v>37.506999999997788</v>
       </c>
       <c r="I106" s="7">
-        <f>IF(F106=0,0,H106/F106)</f>
+        <f t="shared" si="7"/>
         <v>3.5266664672040879E-4</v>
       </c>
     </row>
@@ -5509,11 +5506,11 @@
         <v>129352.883</v>
       </c>
       <c r="H107" s="6">
-        <f>G107-F107</f>
+        <f t="shared" si="6"/>
         <v>45.445000000006985</v>
       </c>
       <c r="I107" s="7">
-        <f>IF(F107=0,0,H107/F107)</f>
+        <f t="shared" si="7"/>
         <v>3.5144923372472191E-4</v>
       </c>
     </row>
@@ -5540,11 +5537,11 @@
         <v>33024.42</v>
       </c>
       <c r="H108" s="6">
-        <f>G108-F108</f>
+        <f t="shared" si="6"/>
         <v>11.582999999998719</v>
       </c>
       <c r="I108" s="7">
-        <f>IF(F108=0,0,H108/F108)</f>
+        <f t="shared" si="7"/>
         <v>3.5086351409297905E-4</v>
       </c>
     </row>
@@ -5571,11 +5568,11 @@
         <v>541753.20200000005</v>
       </c>
       <c r="H109" s="6">
-        <f>G109-F109</f>
+        <f t="shared" si="6"/>
         <v>189.11499999999069</v>
       </c>
       <c r="I109" s="7">
-        <f>IF(F109=0,0,H109/F109)</f>
+        <f t="shared" si="7"/>
         <v>3.4920151564627415E-4</v>
       </c>
     </row>
@@ -5602,11 +5599,11 @@
         <v>331808.70699999999</v>
       </c>
       <c r="H110" s="6">
-        <f>G110-F110</f>
+        <f t="shared" si="6"/>
         <v>115.76600000000326</v>
       </c>
       <c r="I110" s="7">
-        <f>IF(F110=0,0,H110/F110)</f>
+        <f t="shared" si="7"/>
         <v>3.4901556738285624E-4</v>
       </c>
     </row>
@@ -5633,11 +5630,11 @@
         <v>37386.029000000002</v>
       </c>
       <c r="H111" s="6">
-        <f>G111-F111</f>
+        <f t="shared" si="6"/>
         <v>13.041000000004715</v>
       </c>
       <c r="I111" s="7">
-        <f>IF(F111=0,0,H111/F111)</f>
+        <f t="shared" si="7"/>
         <v>3.489418614322386E-4</v>
       </c>
     </row>
@@ -5664,11 +5661,11 @@
         <v>10983.181</v>
       </c>
       <c r="H112" s="6">
-        <f>G112-F112</f>
+        <f t="shared" si="6"/>
         <v>3.816000000000713</v>
       </c>
       <c r="I112" s="7">
-        <f>IF(F112=0,0,H112/F112)</f>
+        <f t="shared" si="7"/>
         <v>3.4756108390610139E-4</v>
       </c>
     </row>
@@ -5695,11 +5692,11 @@
         <v>149054.03700000001</v>
       </c>
       <c r="H113" s="6">
-        <f>G113-F113</f>
+        <f t="shared" si="6"/>
         <v>51.583000000013271</v>
       </c>
       <c r="I113" s="7">
-        <f>IF(F113=0,0,H113/F113)</f>
+        <f t="shared" si="7"/>
         <v>3.4618892921061068E-4</v>
       </c>
     </row>
@@ -5726,11 +5723,11 @@
         <v>30870.053</v>
       </c>
       <c r="H114" s="6">
-        <f>G114-F114</f>
+        <f t="shared" si="6"/>
         <v>10.641999999999825</v>
       </c>
       <c r="I114" s="7">
-        <f>IF(F114=0,0,H114/F114)</f>
+        <f t="shared" si="7"/>
         <v>3.4485428124340499E-4</v>
       </c>
     </row>
@@ -5757,11 +5754,11 @@
         <v>22399.794000000002</v>
       </c>
       <c r="H115" s="6">
-        <f>G115-F115</f>
+        <f t="shared" si="6"/>
         <v>7.7040000000015425</v>
       </c>
       <c r="I115" s="7">
-        <f>IF(F115=0,0,H115/F115)</f>
+        <f t="shared" si="7"/>
         <v>3.4405006410752825E-4</v>
       </c>
     </row>
@@ -5788,11 +5785,11 @@
         <v>28631.383000000002</v>
       </c>
       <c r="H116" s="6">
-        <f>G116-F116</f>
+        <f t="shared" si="6"/>
         <v>9.8370000000031723</v>
       </c>
       <c r="I116" s="7">
-        <f>IF(F116=0,0,H116/F116)</f>
+        <f t="shared" si="7"/>
         <v>3.4369212620461429E-4</v>
       </c>
     </row>
@@ -5819,11 +5816,11 @@
         <v>209214.46100000001</v>
       </c>
       <c r="H117" s="6">
-        <f>G117-F117</f>
+        <f t="shared" si="6"/>
         <v>71.774000000004889</v>
       </c>
       <c r="I117" s="7">
-        <f>IF(F117=0,0,H117/F117)</f>
+        <f t="shared" si="7"/>
         <v>3.431819731760685E-4</v>
       </c>
     </row>
@@ -5850,11 +5847,11 @@
         <v>74122.764999999999</v>
       </c>
       <c r="H118" s="6">
-        <f>G118-F118</f>
+        <f t="shared" si="6"/>
         <v>25.375</v>
       </c>
       <c r="I118" s="7">
-        <f>IF(F118=0,0,H118/F118)</f>
+        <f t="shared" si="7"/>
         <v>3.424547072440743E-4</v>
       </c>
     </row>
@@ -5881,11 +5878,11 @@
         <v>190835.916</v>
       </c>
       <c r="H119" s="6">
-        <f>G119-F119</f>
+        <f t="shared" si="6"/>
         <v>65.24900000001071</v>
       </c>
       <c r="I119" s="7">
-        <f>IF(F119=0,0,H119/F119)</f>
+        <f t="shared" si="7"/>
         <v>3.4202847338165839E-4</v>
       </c>
     </row>
@@ -5912,11 +5909,11 @@
         <v>246415.29500000001</v>
       </c>
       <c r="H120" s="6">
-        <f>G120-F120</f>
+        <f t="shared" si="6"/>
         <v>84.221000000019558</v>
       </c>
       <c r="I120" s="7">
-        <f>IF(F120=0,0,H120/F120)</f>
+        <f t="shared" si="7"/>
         <v>3.4190164737405218E-4</v>
       </c>
     </row>
@@ -5943,11 +5940,11 @@
         <v>159215.41699999999</v>
       </c>
       <c r="H121" s="6">
-        <f>G121-F121</f>
+        <f t="shared" si="6"/>
         <v>54.237999999983003</v>
       </c>
       <c r="I121" s="7">
-        <f>IF(F121=0,0,H121/F121)</f>
+        <f t="shared" si="7"/>
         <v>3.4077405269775617E-4</v>
       </c>
     </row>
@@ -5974,11 +5971,11 @@
         <v>199570.04300000001</v>
       </c>
       <c r="H122" s="6">
-        <f>G122-F122</f>
+        <f t="shared" si="6"/>
         <v>67.940000000002328</v>
       </c>
       <c r="I122" s="7">
-        <f>IF(F122=0,0,H122/F122)</f>
+        <f t="shared" si="7"/>
         <v>3.4054778861154322E-4</v>
       </c>
     </row>
@@ -6005,11 +6002,11 @@
         <v>52848.504000000001</v>
       </c>
       <c r="H123" s="6">
-        <f>G123-F123</f>
+        <f t="shared" si="6"/>
         <v>17.950000000004366</v>
       </c>
       <c r="I123" s="7">
-        <f>IF(F123=0,0,H123/F123)</f>
+        <f t="shared" si="7"/>
         <v>3.3976550766445432E-4</v>
       </c>
     </row>
@@ -6036,11 +6033,11 @@
         <v>62908.735000000001</v>
       </c>
       <c r="H124" s="6">
-        <f>G124-F124</f>
+        <f t="shared" si="6"/>
         <v>21.357000000003609</v>
       </c>
       <c r="I124" s="7">
-        <f>IF(F124=0,0,H124/F124)</f>
+        <f t="shared" si="7"/>
         <v>3.3960709889993519E-4</v>
       </c>
     </row>
@@ -6067,11 +6064,11 @@
         <v>14479.947</v>
       </c>
       <c r="H125" s="6">
-        <f>G125-F125</f>
+        <f t="shared" si="6"/>
         <v>4.9050000000006548</v>
       </c>
       <c r="I125" s="7">
-        <f>IF(F125=0,0,H125/F125)</f>
+        <f t="shared" si="7"/>
         <v>3.3885912040881503E-4</v>
       </c>
     </row>
@@ -6098,11 +6095,11 @@
         <v>62825.953000000001</v>
       </c>
       <c r="H126" s="6">
-        <f>G126-F126</f>
+        <f t="shared" si="6"/>
         <v>21.279999999998836</v>
       </c>
       <c r="I126" s="7">
-        <f>IF(F126=0,0,H126/F126)</f>
+        <f t="shared" si="7"/>
         <v>3.3882829069102605E-4</v>
       </c>
     </row>
@@ -6129,11 +6126,11 @@
         <v>34221.762000000002</v>
       </c>
       <c r="H127" s="6">
-        <f>G127-F127</f>
+        <f t="shared" si="6"/>
         <v>11.583000000005995</v>
       </c>
       <c r="I127" s="7">
-        <f>IF(F127=0,0,H127/F127)</f>
+        <f t="shared" si="7"/>
         <v>3.3858343740341134E-4</v>
       </c>
     </row>
@@ -6160,11 +6157,11 @@
         <v>445020.29700000002</v>
       </c>
       <c r="H128" s="6">
-        <f>G128-F128</f>
+        <f t="shared" si="6"/>
         <v>150.59500000003027</v>
       </c>
       <c r="I128" s="7">
-        <f>IF(F128=0,0,H128/F128)</f>
+        <f t="shared" si="7"/>
         <v>3.3851484900635078E-4</v>
       </c>
     </row>
@@ -6191,11 +6188,11 @@
         <v>409693.06599999999</v>
       </c>
       <c r="H129" s="6">
-        <f>G129-F129</f>
+        <f t="shared" si="6"/>
         <v>138.56699999998091</v>
       </c>
       <c r="I129" s="7">
-        <f>IF(F129=0,0,H129/F129)</f>
+        <f t="shared" si="7"/>
         <v>3.3833592437225527E-4</v>
       </c>
     </row>
@@ -6222,11 +6219,11 @@
         <v>509983.065</v>
       </c>
       <c r="H130" s="6">
-        <f>G130-F130</f>
+        <f t="shared" ref="H130:H161" si="8">G130-F130</f>
         <v>171.11099999997532</v>
       </c>
       <c r="I130" s="7">
-        <f>IF(F130=0,0,H130/F130)</f>
+        <f t="shared" ref="I130:I161" si="9">IF(F130=0,0,H130/F130)</f>
         <v>3.3563551944483299E-4</v>
       </c>
     </row>
@@ -6253,11 +6250,11 @@
         <v>118752.75199999999</v>
       </c>
       <c r="H131" s="6">
-        <f>G131-F131</f>
+        <f t="shared" si="8"/>
         <v>39.783999999999651</v>
       </c>
       <c r="I131" s="7">
-        <f>IF(F131=0,0,H131/F131)</f>
+        <f t="shared" si="9"/>
         <v>3.3512766692851665E-4</v>
       </c>
     </row>
@@ -6284,11 +6281,11 @@
         <v>79312.210000000006</v>
       </c>
       <c r="H132" s="6">
-        <f>G132-F132</f>
+        <f t="shared" si="8"/>
         <v>26.55000000000291</v>
       </c>
       <c r="I132" s="7">
-        <f>IF(F132=0,0,H132/F132)</f>
+        <f t="shared" si="9"/>
         <v>3.3486509414190293E-4</v>
       </c>
     </row>
@@ -6315,11 +6312,11 @@
         <v>117728.871</v>
       </c>
       <c r="H133" s="6">
-        <f>G133-F133</f>
+        <f t="shared" si="8"/>
         <v>39.406000000002678</v>
       </c>
       <c r="I133" s="7">
-        <f>IF(F133=0,0,H133/F133)</f>
+        <f t="shared" si="9"/>
         <v>3.3483030957785965E-4</v>
       </c>
     </row>
@@ -6346,11 +6343,11 @@
         <v>371933.413</v>
       </c>
       <c r="H134" s="6">
-        <f>G134-F134</f>
+        <f t="shared" si="8"/>
         <v>124.38299999997253</v>
       </c>
       <c r="I134" s="7">
-        <f>IF(F134=0,0,H134/F134)</f>
+        <f t="shared" si="9"/>
         <v>3.3453464000046614E-4</v>
       </c>
     </row>
@@ -6377,11 +6374,11 @@
         <v>93262.615999999995</v>
       </c>
       <c r="H135" s="6">
-        <f>G135-F135</f>
+        <f t="shared" si="8"/>
         <v>31.161999999996624</v>
       </c>
       <c r="I135" s="7">
-        <f>IF(F135=0,0,H135/F135)</f>
+        <f t="shared" si="9"/>
         <v>3.3424341960811449E-4</v>
       </c>
     </row>
@@ -6408,11 +6405,11 @@
         <v>137226.467</v>
       </c>
       <c r="H136" s="6">
-        <f>G136-F136</f>
+        <f t="shared" si="8"/>
         <v>45.724000000016531</v>
       </c>
       <c r="I136" s="7">
-        <f>IF(F136=0,0,H136/F136)</f>
+        <f t="shared" si="9"/>
         <v>3.3331208885504094E-4</v>
       </c>
     </row>
@@ -6439,11 +6436,11 @@
         <v>74568.687000000005</v>
       </c>
       <c r="H137" s="6">
-        <f>G137-F137</f>
+        <f t="shared" si="8"/>
         <v>24.804000000003725</v>
       </c>
       <c r="I137" s="7">
-        <f>IF(F137=0,0,H137/F137)</f>
+        <f t="shared" si="9"/>
         <v>3.3274360016909404E-4</v>
       </c>
     </row>
@@ -6470,11 +6467,11 @@
         <v>90641.849000000002</v>
       </c>
       <c r="H138" s="6">
-        <f>G138-F138</f>
+        <f t="shared" si="8"/>
         <v>29.964999999996508</v>
       </c>
       <c r="I138" s="7">
-        <f>IF(F138=0,0,H138/F138)</f>
+        <f t="shared" si="9"/>
         <v>3.3069613694376455E-4</v>
       </c>
     </row>
@@ -6501,11 +6498,11 @@
         <v>35224.125</v>
       </c>
       <c r="H139" s="6">
-        <f>G139-F139</f>
+        <f t="shared" si="8"/>
         <v>11.637000000002445</v>
       </c>
       <c r="I139" s="7">
-        <f>IF(F139=0,0,H139/F139)</f>
+        <f t="shared" si="9"/>
         <v>3.3047934585032576E-4</v>
       </c>
     </row>
@@ -6532,11 +6529,11 @@
         <v>365971.26400000002</v>
       </c>
       <c r="H140" s="6">
-        <f>G140-F140</f>
+        <f t="shared" si="8"/>
         <v>120.79200000001583</v>
       </c>
       <c r="I140" s="7">
-        <f>IF(F140=0,0,H140/F140)</f>
+        <f t="shared" si="9"/>
         <v>3.301676757164764E-4</v>
       </c>
     </row>
@@ -6563,11 +6560,11 @@
         <v>27888.367999999999</v>
       </c>
       <c r="H141" s="6">
-        <f>G141-F141</f>
+        <f t="shared" si="8"/>
         <v>9.1980000000003201</v>
       </c>
       <c r="I141" s="7">
-        <f>IF(F141=0,0,H141/F141)</f>
+        <f t="shared" si="9"/>
         <v>3.299237387626791E-4</v>
       </c>
     </row>
@@ -6594,11 +6591,11 @@
         <v>24777.339</v>
       </c>
       <c r="H142" s="6">
-        <f>G142-F142</f>
+        <f t="shared" si="8"/>
         <v>8.1630000000004657</v>
       </c>
       <c r="I142" s="7">
-        <f>IF(F142=0,0,H142/F142)</f>
+        <f t="shared" si="9"/>
         <v>3.2956284052406369E-4</v>
       </c>
     </row>
@@ -6625,11 +6622,11 @@
         <v>56483.381999999998</v>
       </c>
       <c r="H143" s="6">
-        <f>G143-F143</f>
+        <f t="shared" si="8"/>
         <v>18.588999999999942</v>
       </c>
       <c r="I143" s="7">
-        <f>IF(F143=0,0,H143/F143)</f>
+        <f t="shared" si="9"/>
         <v>3.2921399357649188E-4</v>
       </c>
     </row>
@@ -6656,11 +6653,11 @@
         <v>24245.832999999999</v>
       </c>
       <c r="H144" s="6">
-        <f>G144-F144</f>
+        <f t="shared" si="8"/>
         <v>7.9470000000001164</v>
       </c>
       <c r="I144" s="7">
-        <f>IF(F144=0,0,H144/F144)</f>
+        <f t="shared" si="9"/>
         <v>3.2787512904384965E-4</v>
       </c>
     </row>
@@ -6687,11 +6684,11 @@
         <v>13654.513999999999</v>
       </c>
       <c r="H145" s="6">
-        <f>G145-F145</f>
+        <f t="shared" si="8"/>
         <v>4.4459999999999127</v>
       </c>
       <c r="I145" s="7">
-        <f>IF(F145=0,0,H145/F145)</f>
+        <f t="shared" si="9"/>
         <v>3.2571266311639716E-4</v>
       </c>
     </row>
@@ -6718,11 +6715,11 @@
         <v>25651.161</v>
       </c>
       <c r="H146" s="6">
-        <f>G146-F146</f>
+        <f t="shared" si="8"/>
         <v>8.1270000000004075</v>
       </c>
       <c r="I146" s="7">
-        <f>IF(F146=0,0,H146/F146)</f>
+        <f t="shared" si="9"/>
         <v>3.1692817628368032E-4</v>
       </c>
     </row>
@@ -6805,11 +6802,11 @@
         <v>1</v>
       </c>
       <c r="H2" s="6">
-        <f>F2-G2</f>
+        <f t="shared" ref="H2:H65" si="0">F2-G2</f>
         <v>146021</v>
       </c>
       <c r="I2" s="7">
-        <f>IF(F2=0,0,H2/F2)</f>
+        <f t="shared" ref="I2:I65" si="1">IF(F2=0,0,H2/F2)</f>
         <v>0.99999315171686454</v>
       </c>
     </row>
@@ -6836,11 +6833,11 @@
         <v>1</v>
       </c>
       <c r="H3" s="6">
-        <f>F3-G3</f>
+        <f t="shared" si="0"/>
         <v>57949</v>
       </c>
       <c r="I3" s="7">
-        <f>IF(F3=0,0,H3/F3)</f>
+        <f t="shared" si="1"/>
         <v>0.99998274374460738</v>
       </c>
     </row>
@@ -6867,11 +6864,11 @@
         <v>899717</v>
       </c>
       <c r="H4" s="6">
-        <f>F4-G4</f>
+        <f t="shared" si="0"/>
         <v>19300</v>
       </c>
       <c r="I4" s="7">
-        <f>IF(F4=0,0,H4/F4)</f>
+        <f t="shared" si="1"/>
         <v>2.1000699660615636E-2</v>
       </c>
     </row>
@@ -6898,11 +6895,11 @@
         <v>1</v>
       </c>
       <c r="H5" s="6">
-        <f>F5-G5</f>
+        <f t="shared" si="0"/>
         <v>17939</v>
       </c>
       <c r="I5" s="7">
-        <f>IF(F5=0,0,H5/F5)</f>
+        <f t="shared" si="1"/>
         <v>0.99994425863991077</v>
       </c>
     </row>
@@ -6929,11 +6926,11 @@
         <v>0.441</v>
       </c>
       <c r="H6" s="6">
-        <f>F6-G6</f>
+        <f t="shared" si="0"/>
         <v>15212</v>
       </c>
       <c r="I6" s="7">
-        <f>IF(F6=0,0,H6/F6)</f>
+        <f t="shared" si="1"/>
         <v>0.9999710105695726</v>
       </c>
     </row>
@@ -6960,11 +6957,11 @@
         <v>1</v>
       </c>
       <c r="H7" s="6">
-        <f>F7-G7</f>
+        <f t="shared" si="0"/>
         <v>12599</v>
       </c>
       <c r="I7" s="7">
-        <f>IF(F7=0,0,H7/F7)</f>
+        <f t="shared" si="1"/>
         <v>0.99992063492063488</v>
       </c>
     </row>
@@ -6991,11 +6988,11 @@
         <v>1</v>
       </c>
       <c r="H8" s="6">
-        <f>F8-G8</f>
+        <f t="shared" si="0"/>
         <v>11039</v>
       </c>
       <c r="I8" s="7">
-        <f>IF(F8=0,0,H8/F8)</f>
+        <f t="shared" si="1"/>
         <v>0.99990942028985508</v>
       </c>
     </row>
@@ -7022,11 +7019,11 @@
         <v>1</v>
       </c>
       <c r="H9" s="6">
-        <f>F9-G9</f>
+        <f t="shared" si="0"/>
         <v>10770</v>
       </c>
       <c r="I9" s="7">
-        <f>IF(F9=0,0,H9/F9)</f>
+        <f t="shared" si="1"/>
         <v>0.99990715810973907</v>
       </c>
     </row>
@@ -7053,11 +7050,11 @@
         <v>1</v>
       </c>
       <c r="H10" s="6">
-        <f>F10-G10</f>
+        <f t="shared" si="0"/>
         <v>10019</v>
       </c>
       <c r="I10" s="7">
-        <f>IF(F10=0,0,H10/F10)</f>
+        <f t="shared" si="1"/>
         <v>0.99990019960079846</v>
       </c>
     </row>
@@ -7084,11 +7081,11 @@
         <v>269844</v>
       </c>
       <c r="H11" s="6">
-        <f>F11-G11</f>
+        <f t="shared" si="0"/>
         <v>9590</v>
       </c>
       <c r="I11" s="7">
-        <f>IF(F11=0,0,H11/F11)</f>
+        <f t="shared" si="1"/>
         <v>3.4319374163487619E-2</v>
       </c>
     </row>
@@ -7115,11 +7112,11 @@
         <v>1</v>
       </c>
       <c r="H12" s="6">
-        <f>F12-G12</f>
+        <f t="shared" si="0"/>
         <v>9273</v>
       </c>
       <c r="I12" s="7">
-        <f>IF(F12=0,0,H12/F12)</f>
+        <f t="shared" si="1"/>
         <v>0.99989217166271294</v>
       </c>
     </row>
@@ -7146,11 +7143,11 @@
         <v>1</v>
       </c>
       <c r="H13" s="6">
-        <f>F13-G13</f>
+        <f t="shared" si="0"/>
         <v>6979</v>
       </c>
       <c r="I13" s="7">
-        <f>IF(F13=0,0,H13/F13)</f>
+        <f t="shared" si="1"/>
         <v>0.99985673352435533</v>
       </c>
     </row>
@@ -7177,11 +7174,11 @@
         <v>1</v>
       </c>
       <c r="H14" s="6">
-        <f>F14-G14</f>
+        <f t="shared" si="0"/>
         <v>6815</v>
       </c>
       <c r="I14" s="7">
-        <f>IF(F14=0,0,H14/F14)</f>
+        <f t="shared" si="1"/>
         <v>0.9998532863849765</v>
       </c>
     </row>
@@ -7208,11 +7205,11 @@
         <v>1</v>
       </c>
       <c r="H15" s="6">
-        <f>F15-G15</f>
+        <f t="shared" si="0"/>
         <v>6699</v>
       </c>
       <c r="I15" s="7">
-        <f>IF(F15=0,0,H15/F15)</f>
+        <f t="shared" si="1"/>
         <v>0.99985074626865666</v>
       </c>
     </row>
@@ -7239,11 +7236,11 @@
         <v>667080</v>
       </c>
       <c r="H16" s="6">
-        <f>F16-G16</f>
+        <f t="shared" si="0"/>
         <v>5270</v>
       </c>
       <c r="I16" s="7">
-        <f>IF(F16=0,0,H16/F16)</f>
+        <f t="shared" si="1"/>
         <v>7.8381795195954489E-3</v>
       </c>
     </row>
@@ -7270,11 +7267,11 @@
         <v>1</v>
       </c>
       <c r="H17" s="6">
-        <f>F17-G17</f>
+        <f t="shared" si="0"/>
         <v>5198</v>
       </c>
       <c r="I17" s="7">
-        <f>IF(F17=0,0,H17/F17)</f>
+        <f t="shared" si="1"/>
         <v>0.99980765531833049</v>
       </c>
     </row>
@@ -7301,11 +7298,11 @@
         <v>37230</v>
       </c>
       <c r="H18" s="6">
-        <f>F18-G18</f>
+        <f t="shared" si="0"/>
         <v>5000</v>
       </c>
       <c r="I18" s="7">
-        <f>IF(F18=0,0,H18/F18)</f>
+        <f t="shared" si="1"/>
         <v>0.11839924224484963</v>
       </c>
     </row>
@@ -7332,11 +7329,11 @@
         <v>1</v>
       </c>
       <c r="H19" s="6">
-        <f>F19-G19</f>
+        <f t="shared" si="0"/>
         <v>4529</v>
       </c>
       <c r="I19" s="7">
-        <f>IF(F19=0,0,H19/F19)</f>
+        <f t="shared" si="1"/>
         <v>0.99977924944812357</v>
       </c>
     </row>
@@ -7363,11 +7360,11 @@
         <v>1</v>
       </c>
       <c r="H20" s="6">
-        <f>F20-G20</f>
+        <f t="shared" si="0"/>
         <v>3409</v>
       </c>
       <c r="I20" s="7">
-        <f>IF(F20=0,0,H20/F20)</f>
+        <f t="shared" si="1"/>
         <v>0.99970674486803524</v>
       </c>
     </row>
@@ -7394,11 +7391,11 @@
         <v>101143</v>
       </c>
       <c r="H21" s="6">
-        <f>F21-G21</f>
+        <f t="shared" si="0"/>
         <v>3280</v>
       </c>
       <c r="I21" s="7">
-        <f>IF(F21=0,0,H21/F21)</f>
+        <f t="shared" si="1"/>
         <v>3.1410704538272223E-2</v>
       </c>
     </row>
@@ -7425,11 +7422,11 @@
         <v>1</v>
       </c>
       <c r="H22" s="6">
-        <f>F22-G22</f>
+        <f t="shared" si="0"/>
         <v>2335</v>
       </c>
       <c r="I22" s="7">
-        <f>IF(F22=0,0,H22/F22)</f>
+        <f t="shared" si="1"/>
         <v>0.99957191780821919</v>
       </c>
     </row>
@@ -7456,11 +7453,11 @@
         <v>1</v>
       </c>
       <c r="H23" s="6">
-        <f>F23-G23</f>
+        <f t="shared" si="0"/>
         <v>1819</v>
       </c>
       <c r="I23" s="7">
-        <f>IF(F23=0,0,H23/F23)</f>
+        <f t="shared" si="1"/>
         <v>0.99945054945054945</v>
       </c>
     </row>
@@ -7487,11 +7484,11 @@
         <v>26430</v>
       </c>
       <c r="H24" s="6">
-        <f>F24-G24</f>
+        <f t="shared" si="0"/>
         <v>1540</v>
       </c>
       <c r="I24" s="7">
-        <f>IF(F24=0,0,H24/F24)</f>
+        <f t="shared" si="1"/>
         <v>5.5058991776903828E-2</v>
       </c>
     </row>
@@ -7518,11 +7515,11 @@
         <v>34700</v>
       </c>
       <c r="H25" s="6">
-        <f>F25-G25</f>
+        <f t="shared" si="0"/>
         <v>1130</v>
       </c>
       <c r="I25" s="7">
-        <f>IF(F25=0,0,H25/F25)</f>
+        <f t="shared" si="1"/>
         <v>3.1537817471392685E-2</v>
       </c>
     </row>
@@ -7549,11 +7546,11 @@
         <v>375900.48599999998</v>
       </c>
       <c r="H26" s="6">
-        <f>F26-G26</f>
+        <f t="shared" si="0"/>
         <v>1108</v>
       </c>
       <c r="I26" s="7">
-        <f>IF(F26=0,0,H26/F26)</f>
+        <f t="shared" si="1"/>
         <v>2.9389258893233509E-3</v>
       </c>
     </row>
@@ -7580,11 +7577,11 @@
         <v>9514</v>
       </c>
       <c r="H27" s="6">
-        <f>F27-G27</f>
+        <f t="shared" si="0"/>
         <v>1000</v>
       </c>
       <c r="I27" s="7">
-        <f>IF(F27=0,0,H27/F27)</f>
+        <f t="shared" si="1"/>
         <v>9.5111280197831466E-2</v>
       </c>
     </row>
@@ -7611,11 +7608,11 @@
         <v>211659</v>
       </c>
       <c r="H28" s="6">
-        <f>F28-G28</f>
+        <f t="shared" si="0"/>
         <v>979</v>
       </c>
       <c r="I28" s="7">
-        <f>IF(F28=0,0,H28/F28)</f>
+        <f t="shared" si="1"/>
         <v>4.6040688870286591E-3</v>
       </c>
     </row>
@@ -7642,11 +7639,11 @@
         <v>28522</v>
       </c>
       <c r="H29" s="6">
-        <f>F29-G29</f>
+        <f t="shared" si="0"/>
         <v>748</v>
       </c>
       <c r="I29" s="7">
-        <f>IF(F29=0,0,H29/F29)</f>
+        <f t="shared" si="1"/>
         <v>2.5555175948069695E-2</v>
       </c>
     </row>
@@ -7673,11 +7670,11 @@
         <v>1</v>
       </c>
       <c r="H30" s="6">
-        <f>F30-G30</f>
+        <f t="shared" si="0"/>
         <v>711</v>
       </c>
       <c r="I30" s="7">
-        <f>IF(F30=0,0,H30/F30)</f>
+        <f t="shared" si="1"/>
         <v>0.9985955056179775</v>
       </c>
     </row>
@@ -7704,11 +7701,11 @@
         <v>226896.516</v>
       </c>
       <c r="H31" s="6">
-        <f>F31-G31</f>
+        <f t="shared" si="0"/>
         <v>670</v>
       </c>
       <c r="I31" s="7">
-        <f>IF(F31=0,0,H31/F31)</f>
+        <f t="shared" si="1"/>
         <v>2.9441941273996566E-3</v>
       </c>
     </row>
@@ -7735,11 +7732,11 @@
         <v>54937</v>
       </c>
       <c r="H32" s="6">
-        <f>F32-G32</f>
+        <f t="shared" si="0"/>
         <v>654</v>
       </c>
       <c r="I32" s="7">
-        <f>IF(F32=0,0,H32/F32)</f>
+        <f t="shared" si="1"/>
         <v>1.1764494252666799E-2</v>
       </c>
     </row>
@@ -7766,11 +7763,11 @@
         <v>20884</v>
       </c>
       <c r="H33" s="6">
-        <f>F33-G33</f>
+        <f t="shared" si="0"/>
         <v>643</v>
       </c>
       <c r="I33" s="7">
-        <f>IF(F33=0,0,H33/F33)</f>
+        <f t="shared" si="1"/>
         <v>2.9869466251683931E-2</v>
       </c>
     </row>
@@ -7797,11 +7794,11 @@
         <v>69670</v>
       </c>
       <c r="H34" s="6">
-        <f>F34-G34</f>
+        <f t="shared" si="0"/>
         <v>631</v>
       </c>
       <c r="I34" s="7">
-        <f>IF(F34=0,0,H34/F34)</f>
+        <f t="shared" si="1"/>
         <v>8.9756902462269379E-3</v>
       </c>
     </row>
@@ -7828,11 +7825,11 @@
         <v>184975</v>
       </c>
       <c r="H35" s="6">
-        <f>F35-G35</f>
+        <f t="shared" si="0"/>
         <v>546</v>
       </c>
       <c r="I35" s="7">
-        <f>IF(F35=0,0,H35/F35)</f>
+        <f t="shared" si="1"/>
         <v>2.943063049466098E-3</v>
       </c>
     </row>
@@ -7859,11 +7856,11 @@
         <v>15750</v>
       </c>
       <c r="H36" s="6">
-        <f>F36-G36</f>
+        <f t="shared" si="0"/>
         <v>530</v>
       </c>
       <c r="I36" s="7">
-        <f>IF(F36=0,0,H36/F36)</f>
+        <f t="shared" si="1"/>
         <v>3.2555282555282554E-2</v>
       </c>
     </row>
@@ -7890,11 +7887,11 @@
         <v>27329</v>
       </c>
       <c r="H37" s="6">
-        <f>F37-G37</f>
+        <f t="shared" si="0"/>
         <v>450</v>
       </c>
       <c r="I37" s="7">
-        <f>IF(F37=0,0,H37/F37)</f>
+        <f t="shared" si="1"/>
         <v>1.6199287231361822E-2</v>
       </c>
     </row>
@@ -7921,11 +7918,11 @@
         <v>9280</v>
       </c>
       <c r="H38" s="6">
-        <f>F38-G38</f>
+        <f t="shared" si="0"/>
         <v>400</v>
       </c>
       <c r="I38" s="7">
-        <f>IF(F38=0,0,H38/F38)</f>
+        <f t="shared" si="1"/>
         <v>4.1322314049586778E-2</v>
       </c>
     </row>
@@ -7952,11 +7949,11 @@
         <v>134352.94500000001</v>
       </c>
       <c r="H39" s="6">
-        <f>F39-G39</f>
+        <f t="shared" si="0"/>
         <v>397</v>
       </c>
       <c r="I39" s="7">
-        <f>IF(F39=0,0,H39/F39)</f>
+        <f t="shared" si="1"/>
         <v>2.9461978630121147E-3</v>
       </c>
     </row>
@@ -7983,11 +7980,11 @@
         <v>43220</v>
       </c>
       <c r="H40" s="6">
-        <f>F40-G40</f>
+        <f t="shared" si="0"/>
         <v>276</v>
       </c>
       <c r="I40" s="7">
-        <f>IF(F40=0,0,H40/F40)</f>
+        <f t="shared" si="1"/>
         <v>6.3454110722825086E-3</v>
       </c>
     </row>
@@ -8014,11 +8011,11 @@
         <v>34668</v>
       </c>
       <c r="H41" s="6">
-        <f>F41-G41</f>
+        <f t="shared" si="0"/>
         <v>269</v>
       </c>
       <c r="I41" s="7">
-        <f>IF(F41=0,0,H41/F41)</f>
+        <f t="shared" si="1"/>
         <v>7.6995735180467699E-3</v>
       </c>
     </row>
@@ -8045,11 +8042,11 @@
         <v>9073</v>
       </c>
       <c r="H42" s="6">
-        <f>F42-G42</f>
+        <f t="shared" si="0"/>
         <v>256</v>
       </c>
       <c r="I42" s="7">
-        <f>IF(F42=0,0,H42/F42)</f>
+        <f t="shared" si="1"/>
         <v>2.7441312037731803E-2</v>
       </c>
     </row>
@@ -8076,11 +8073,11 @@
         <v>42512</v>
       </c>
       <c r="H43" s="6">
-        <f>F43-G43</f>
+        <f t="shared" si="0"/>
         <v>200</v>
       </c>
       <c r="I43" s="7">
-        <f>IF(F43=0,0,H43/F43)</f>
+        <f t="shared" si="1"/>
         <v>4.6825248173815318E-3</v>
       </c>
     </row>
@@ -8107,11 +8104,11 @@
         <v>28779</v>
       </c>
       <c r="H44" s="6">
-        <f>F44-G44</f>
+        <f t="shared" si="0"/>
         <v>194</v>
       </c>
       <c r="I44" s="7">
-        <f>IF(F44=0,0,H44/F44)</f>
+        <f t="shared" si="1"/>
         <v>6.6958892762226897E-3</v>
       </c>
     </row>
@@ -8138,11 +8135,11 @@
         <v>28448</v>
       </c>
       <c r="H45" s="6">
-        <f>F45-G45</f>
+        <f t="shared" si="0"/>
         <v>193</v>
       </c>
       <c r="I45" s="7">
-        <f>IF(F45=0,0,H45/F45)</f>
+        <f t="shared" si="1"/>
         <v>6.7385915296253622E-3</v>
       </c>
     </row>
@@ -8169,11 +8166,11 @@
         <v>62491</v>
       </c>
       <c r="H46" s="6">
-        <f>F46-G46</f>
+        <f t="shared" si="0"/>
         <v>184</v>
       </c>
       <c r="I46" s="7">
-        <f>IF(F46=0,0,H46/F46)</f>
+        <f t="shared" si="1"/>
         <v>2.9357798165137615E-3</v>
       </c>
     </row>
@@ -8200,11 +8197,11 @@
         <v>17508</v>
       </c>
       <c r="H47" s="6">
-        <f>F47-G47</f>
+        <f t="shared" si="0"/>
         <v>182</v>
       </c>
       <c r="I47" s="7">
-        <f>IF(F47=0,0,H47/F47)</f>
+        <f t="shared" si="1"/>
         <v>1.0288298473713963E-2</v>
       </c>
     </row>
@@ -8231,11 +8228,11 @@
         <v>5647</v>
       </c>
       <c r="H48" s="6">
-        <f>F48-G48</f>
+        <f t="shared" si="0"/>
         <v>173</v>
       </c>
       <c r="I48" s="7">
-        <f>IF(F48=0,0,H48/F48)</f>
+        <f t="shared" si="1"/>
         <v>2.9725085910652919E-2</v>
       </c>
     </row>
@@ -8262,11 +8259,11 @@
         <v>9295</v>
       </c>
       <c r="H49" s="6">
-        <f>F49-G49</f>
+        <f t="shared" si="0"/>
         <v>169</v>
       </c>
       <c r="I49" s="7">
-        <f>IF(F49=0,0,H49/F49)</f>
+        <f t="shared" si="1"/>
         <v>1.7857142857142856E-2</v>
       </c>
     </row>
@@ -8293,11 +8290,11 @@
         <v>37817</v>
       </c>
       <c r="H50" s="6">
-        <f>F50-G50</f>
+        <f t="shared" si="0"/>
         <v>152</v>
       </c>
       <c r="I50" s="7">
-        <f>IF(F50=0,0,H50/F50)</f>
+        <f t="shared" si="1"/>
         <v>4.0032658221180436E-3</v>
       </c>
     </row>
@@ -8324,11 +8321,11 @@
         <v>41365</v>
       </c>
       <c r="H51" s="6">
-        <f>F51-G51</f>
+        <f t="shared" si="0"/>
         <v>124</v>
       </c>
       <c r="I51" s="7">
-        <f>IF(F51=0,0,H51/F51)</f>
+        <f t="shared" si="1"/>
         <v>2.9887440044349105E-3</v>
       </c>
     </row>
@@ -8355,11 +8352,11 @@
         <v>2920</v>
       </c>
       <c r="H52" s="6">
-        <f>F52-G52</f>
+        <f t="shared" si="0"/>
         <v>115</v>
       </c>
       <c r="I52" s="7">
-        <f>IF(F52=0,0,H52/F52)</f>
+        <f t="shared" si="1"/>
         <v>3.789126853377265E-2</v>
       </c>
     </row>
@@ -8386,11 +8383,11 @@
         <v>2540.596</v>
       </c>
       <c r="H53" s="6">
-        <f>F53-G53</f>
+        <f t="shared" si="0"/>
         <v>108.31399999999985</v>
       </c>
       <c r="I53" s="7">
-        <f>IF(F53=0,0,H53/F53)</f>
+        <f t="shared" si="1"/>
         <v>4.0890026463715208E-2</v>
       </c>
     </row>
@@ -8417,11 +8414,11 @@
         <v>7586</v>
       </c>
       <c r="H54" s="6">
-        <f>F54-G54</f>
+        <f t="shared" si="0"/>
         <v>101</v>
       </c>
       <c r="I54" s="7">
-        <f>IF(F54=0,0,H54/F54)</f>
+        <f t="shared" si="1"/>
         <v>1.3139065955509302E-2</v>
       </c>
     </row>
@@ -8448,11 +8445,11 @@
         <v>19487</v>
       </c>
       <c r="H55" s="6">
-        <f>F55-G55</f>
+        <f t="shared" si="0"/>
         <v>100</v>
       </c>
       <c r="I55" s="7">
-        <f>IF(F55=0,0,H55/F55)</f>
+        <f t="shared" si="1"/>
         <v>5.1054270689743194E-3</v>
       </c>
     </row>
@@ -8479,11 +8476,11 @@
         <v>7400</v>
       </c>
       <c r="H56" s="6">
-        <f>F56-G56</f>
+        <f t="shared" si="0"/>
         <v>100</v>
       </c>
       <c r="I56" s="7">
-        <f>IF(F56=0,0,H56/F56)</f>
+        <f t="shared" si="1"/>
         <v>1.3333333333333334E-2</v>
       </c>
     </row>
@@ -8510,11 +8507,11 @@
         <v>9778.5499999999993</v>
       </c>
       <c r="H57" s="6">
-        <f>F57-G57</f>
+        <f t="shared" si="0"/>
         <v>100</v>
       </c>
       <c r="I57" s="7">
-        <f>IF(F57=0,0,H57/F57)</f>
+        <f t="shared" si="1"/>
         <v>1.012294314448983E-2</v>
       </c>
     </row>
@@ -8541,11 +8538,11 @@
         <v>13541</v>
       </c>
       <c r="H58" s="6">
-        <f>F58-G58</f>
+        <f t="shared" si="0"/>
         <v>100</v>
       </c>
       <c r="I58" s="7">
-        <f>IF(F58=0,0,H58/F58)</f>
+        <f t="shared" si="1"/>
         <v>7.3308408474452016E-3</v>
       </c>
     </row>
@@ -8572,11 +8569,11 @@
         <v>15322.04</v>
       </c>
       <c r="H59" s="6">
-        <f>F59-G59</f>
+        <f t="shared" si="0"/>
         <v>100</v>
       </c>
       <c r="I59" s="7">
-        <f>IF(F59=0,0,H59/F59)</f>
+        <f t="shared" si="1"/>
         <v>6.4842264706874058E-3</v>
       </c>
     </row>
@@ -8603,11 +8600,11 @@
         <v>20465</v>
       </c>
       <c r="H60" s="6">
-        <f>F60-G60</f>
+        <f t="shared" si="0"/>
         <v>100</v>
       </c>
       <c r="I60" s="7">
-        <f>IF(F60=0,0,H60/F60)</f>
+        <f t="shared" si="1"/>
         <v>4.8626306831996112E-3</v>
       </c>
     </row>
@@ -8634,11 +8631,11 @@
         <v>165</v>
       </c>
       <c r="H61" s="6">
-        <f>F61-G61</f>
+        <f t="shared" si="0"/>
         <v>98</v>
       </c>
       <c r="I61" s="7">
-        <f>IF(F61=0,0,H61/F61)</f>
+        <f t="shared" si="1"/>
         <v>0.37262357414448671</v>
       </c>
     </row>
@@ -8665,11 +8662,11 @@
         <v>25907</v>
       </c>
       <c r="H62" s="6">
-        <f>F62-G62</f>
+        <f t="shared" si="0"/>
         <v>77</v>
       </c>
       <c r="I62" s="7">
-        <f>IF(F62=0,0,H62/F62)</f>
+        <f t="shared" si="1"/>
         <v>2.9633620689655171E-3</v>
       </c>
     </row>
@@ -8696,11 +8693,11 @@
         <v>3753</v>
       </c>
       <c r="H63" s="6">
-        <f>F63-G63</f>
+        <f t="shared" si="0"/>
         <v>71</v>
       </c>
       <c r="I63" s="7">
-        <f>IF(F63=0,0,H63/F63)</f>
+        <f t="shared" si="1"/>
         <v>1.8566945606694561E-2</v>
       </c>
     </row>
@@ -8727,11 +8724,11 @@
         <v>10713</v>
       </c>
       <c r="H64" s="6">
-        <f>F64-G64</f>
+        <f t="shared" si="0"/>
         <v>70</v>
       </c>
       <c r="I64" s="7">
-        <f>IF(F64=0,0,H64/F64)</f>
+        <f t="shared" si="1"/>
         <v>6.4916998979875733E-3</v>
       </c>
     </row>
@@ -8758,11 +8755,11 @@
         <v>4569</v>
       </c>
       <c r="H65" s="6">
-        <f>F65-G65</f>
+        <f t="shared" si="0"/>
         <v>64</v>
       </c>
       <c r="I65" s="7">
-        <f>IF(F65=0,0,H65/F65)</f>
+        <f t="shared" si="1"/>
         <v>1.3813943449169004E-2</v>
       </c>
     </row>
@@ -8789,11 +8786,11 @@
         <v>3370</v>
       </c>
       <c r="H66" s="6">
-        <f>F66-G66</f>
+        <f t="shared" ref="H66:H129" si="2">F66-G66</f>
         <v>60</v>
       </c>
       <c r="I66" s="7">
-        <f>IF(F66=0,0,H66/F66)</f>
+        <f t="shared" ref="I66:I129" si="3">IF(F66=0,0,H66/F66)</f>
         <v>1.7492711370262391E-2</v>
       </c>
     </row>
@@ -8820,11 +8817,11 @@
         <v>2919</v>
       </c>
       <c r="H67" s="6">
-        <f>F67-G67</f>
+        <f t="shared" si="2"/>
         <v>54</v>
       </c>
       <c r="I67" s="7">
-        <f>IF(F67=0,0,H67/F67)</f>
+        <f t="shared" si="3"/>
         <v>1.8163471241170535E-2</v>
       </c>
     </row>
@@ -8851,11 +8848,11 @@
         <v>6398</v>
       </c>
       <c r="H68" s="6">
-        <f>F68-G68</f>
+        <f t="shared" si="2"/>
         <v>50</v>
       </c>
       <c r="I68" s="7">
-        <f>IF(F68=0,0,H68/F68)</f>
+        <f t="shared" si="3"/>
         <v>7.7543424317617869E-3</v>
       </c>
     </row>
@@ -8882,11 +8879,11 @@
         <v>6184</v>
       </c>
       <c r="H69" s="6">
-        <f>F69-G69</f>
+        <f t="shared" si="2"/>
         <v>50</v>
       </c>
       <c r="I69" s="7">
-        <f>IF(F69=0,0,H69/F69)</f>
+        <f t="shared" si="3"/>
         <v>8.0205325633622079E-3</v>
       </c>
     </row>
@@ -8913,11 +8910,11 @@
         <v>16805</v>
       </c>
       <c r="H70" s="6">
-        <f>F70-G70</f>
+        <f t="shared" si="2"/>
         <v>50</v>
       </c>
       <c r="I70" s="7">
-        <f>IF(F70=0,0,H70/F70)</f>
+        <f t="shared" si="3"/>
         <v>2.9664787896766538E-3</v>
       </c>
     </row>
@@ -8944,11 +8941,11 @@
         <v>5540</v>
       </c>
       <c r="H71" s="6">
-        <f>F71-G71</f>
+        <f t="shared" si="2"/>
         <v>50</v>
       </c>
       <c r="I71" s="7">
-        <f>IF(F71=0,0,H71/F71)</f>
+        <f t="shared" si="3"/>
         <v>8.9445438282647581E-3</v>
       </c>
     </row>
@@ -8975,11 +8972,11 @@
         <v>4943.0730000000003</v>
       </c>
       <c r="H72" s="6">
-        <f>F72-G72</f>
+        <f t="shared" si="2"/>
         <v>45</v>
       </c>
       <c r="I72" s="7">
-        <f>IF(F72=0,0,H72/F72)</f>
+        <f t="shared" si="3"/>
         <v>9.0215199336497274E-3</v>
       </c>
     </row>
@@ -9006,11 +9003,11 @@
         <v>299</v>
       </c>
       <c r="H73" s="6">
-        <f>F73-G73</f>
+        <f t="shared" si="2"/>
         <v>45</v>
       </c>
       <c r="I73" s="7">
-        <f>IF(F73=0,0,H73/F73)</f>
+        <f t="shared" si="3"/>
         <v>0.1308139534883721</v>
       </c>
     </row>
@@ -9037,11 +9034,11 @@
         <v>2179</v>
       </c>
       <c r="H74" s="6">
-        <f>F74-G74</f>
+        <f t="shared" si="2"/>
         <v>44</v>
       </c>
       <c r="I74" s="7">
-        <f>IF(F74=0,0,H74/F74)</f>
+        <f t="shared" si="3"/>
         <v>1.9793072424651371E-2</v>
       </c>
     </row>
@@ -9068,11 +9065,11 @@
         <v>5614</v>
       </c>
       <c r="H75" s="6">
-        <f>F75-G75</f>
+        <f t="shared" si="2"/>
         <v>38</v>
       </c>
       <c r="I75" s="7">
-        <f>IF(F75=0,0,H75/F75)</f>
+        <f t="shared" si="3"/>
         <v>6.7232837933474876E-3</v>
       </c>
     </row>
@@ -9099,11 +9096,11 @@
         <v>1872</v>
       </c>
       <c r="H76" s="6">
-        <f>F76-G76</f>
+        <f t="shared" si="2"/>
         <v>35</v>
       </c>
       <c r="I76" s="7">
-        <f>IF(F76=0,0,H76/F76)</f>
+        <f t="shared" si="3"/>
         <v>1.8353434714210803E-2</v>
       </c>
     </row>
@@ -9130,11 +9127,11 @@
         <v>5165</v>
       </c>
       <c r="H77" s="6">
-        <f>F77-G77</f>
+        <f t="shared" si="2"/>
         <v>35</v>
       </c>
       <c r="I77" s="7">
-        <f>IF(F77=0,0,H77/F77)</f>
+        <f t="shared" si="3"/>
         <v>6.7307692307692311E-3</v>
       </c>
     </row>
@@ -9161,11 +9158,11 @@
         <v>5229</v>
       </c>
       <c r="H78" s="6">
-        <f>F78-G78</f>
+        <f t="shared" si="2"/>
         <v>35</v>
       </c>
       <c r="I78" s="7">
-        <f>IF(F78=0,0,H78/F78)</f>
+        <f t="shared" si="3"/>
         <v>6.648936170212766E-3</v>
       </c>
     </row>
@@ -9192,11 +9189,11 @@
         <v>4693</v>
       </c>
       <c r="H79" s="6">
-        <f>F79-G79</f>
+        <f t="shared" si="2"/>
         <v>32</v>
       </c>
       <c r="I79" s="7">
-        <f>IF(F79=0,0,H79/F79)</f>
+        <f t="shared" si="3"/>
         <v>6.7724867724867728E-3</v>
       </c>
     </row>
@@ -9223,11 +9220,11 @@
         <v>4352</v>
       </c>
       <c r="H80" s="6">
-        <f>F80-G80</f>
+        <f t="shared" si="2"/>
         <v>30</v>
       </c>
       <c r="I80" s="7">
-        <f>IF(F80=0,0,H80/F80)</f>
+        <f t="shared" si="3"/>
         <v>6.8461889548151527E-3</v>
       </c>
     </row>
@@ -9254,11 +9251,11 @@
         <v>4862</v>
       </c>
       <c r="H81" s="6">
-        <f>F81-G81</f>
+        <f t="shared" si="2"/>
         <v>30</v>
       </c>
       <c r="I81" s="7">
-        <f>IF(F81=0,0,H81/F81)</f>
+        <f t="shared" si="3"/>
         <v>6.1324611610793136E-3</v>
       </c>
     </row>
@@ -9285,11 +9282,11 @@
         <v>3714</v>
       </c>
       <c r="H82" s="6">
-        <f>F82-G82</f>
+        <f t="shared" si="2"/>
         <v>30</v>
       </c>
       <c r="I82" s="7">
-        <f>IF(F82=0,0,H82/F82)</f>
+        <f t="shared" si="3"/>
         <v>8.0128205128205121E-3</v>
       </c>
     </row>
@@ -9316,11 +9313,11 @@
         <v>2934</v>
       </c>
       <c r="H83" s="6">
-        <f>F83-G83</f>
+        <f t="shared" si="2"/>
         <v>29</v>
       </c>
       <c r="I83" s="7">
-        <f>IF(F83=0,0,H83/F83)</f>
+        <f t="shared" si="3"/>
         <v>9.7873776577792771E-3</v>
       </c>
     </row>
@@ -9347,11 +9344,11 @@
         <v>4980</v>
       </c>
       <c r="H84" s="6">
-        <f>F84-G84</f>
+        <f t="shared" si="2"/>
         <v>27</v>
       </c>
       <c r="I84" s="7">
-        <f>IF(F84=0,0,H84/F84)</f>
+        <f t="shared" si="3"/>
         <v>5.3924505692031152E-3</v>
       </c>
     </row>
@@ -9378,11 +9375,11 @@
         <v>3929</v>
       </c>
       <c r="H85" s="6">
-        <f>F85-G85</f>
+        <f t="shared" si="2"/>
         <v>26</v>
       </c>
       <c r="I85" s="7">
-        <f>IF(F85=0,0,H85/F85)</f>
+        <f t="shared" si="3"/>
         <v>6.5739570164348926E-3</v>
       </c>
     </row>
@@ -9409,11 +9406,11 @@
         <v>101591</v>
       </c>
       <c r="H86" s="6">
-        <f>F86-G86</f>
+        <f t="shared" si="2"/>
         <v>25</v>
       </c>
       <c r="I86" s="7">
-        <f>IF(F86=0,0,H86/F86)</f>
+        <f t="shared" si="3"/>
         <v>2.4602424814989767E-4</v>
       </c>
     </row>
@@ -9440,11 +9437,11 @@
         <v>528</v>
       </c>
       <c r="H87" s="6">
-        <f>F87-G87</f>
+        <f t="shared" si="2"/>
         <v>25</v>
       </c>
       <c r="I87" s="7">
-        <f>IF(F87=0,0,H87/F87)</f>
+        <f t="shared" si="3"/>
         <v>4.5207956600361664E-2</v>
       </c>
     </row>
@@ -9471,11 +9468,11 @@
         <v>5024</v>
       </c>
       <c r="H88" s="6">
-        <f>F88-G88</f>
+        <f t="shared" si="2"/>
         <v>22</v>
       </c>
       <c r="I88" s="7">
-        <f>IF(F88=0,0,H88/F88)</f>
+        <f t="shared" si="3"/>
         <v>4.3598890210067376E-3</v>
       </c>
     </row>
@@ -9502,11 +9499,11 @@
         <v>2460</v>
       </c>
       <c r="H89" s="6">
-        <f>F89-G89</f>
+        <f t="shared" si="2"/>
         <v>20</v>
       </c>
       <c r="I89" s="7">
-        <f>IF(F89=0,0,H89/F89)</f>
+        <f t="shared" si="3"/>
         <v>8.0645161290322578E-3</v>
       </c>
     </row>
@@ -9533,11 +9530,11 @@
         <v>1014</v>
       </c>
       <c r="H90" s="6">
-        <f>F90-G90</f>
+        <f t="shared" si="2"/>
         <v>20</v>
       </c>
       <c r="I90" s="7">
-        <f>IF(F90=0,0,H90/F90)</f>
+        <f t="shared" si="3"/>
         <v>1.9342359767891684E-2</v>
       </c>
     </row>
@@ -9564,11 +9561,11 @@
         <v>4654</v>
       </c>
       <c r="H91" s="6">
-        <f>F91-G91</f>
+        <f t="shared" si="2"/>
         <v>20</v>
       </c>
       <c r="I91" s="7">
-        <f>IF(F91=0,0,H91/F91)</f>
+        <f t="shared" si="3"/>
         <v>4.2789901583226361E-3</v>
       </c>
     </row>
@@ -9595,11 +9592,11 @@
         <v>31029</v>
       </c>
       <c r="H92" s="6">
-        <f>F92-G92</f>
+        <f t="shared" si="2"/>
         <v>17</v>
       </c>
       <c r="I92" s="7">
-        <f>IF(F92=0,0,H92/F92)</f>
+        <f t="shared" si="3"/>
         <v>5.4757456677188691E-4</v>
       </c>
     </row>
@@ -9626,11 +9623,11 @@
         <v>27894</v>
       </c>
       <c r="H93" s="6">
-        <f>F93-G93</f>
+        <f t="shared" si="2"/>
         <v>16</v>
       </c>
       <c r="I93" s="7">
-        <f>IF(F93=0,0,H93/F93)</f>
+        <f t="shared" si="3"/>
         <v>5.7327122895019711E-4</v>
       </c>
     </row>
@@ -9657,11 +9654,11 @@
         <v>2448</v>
       </c>
       <c r="H94" s="6">
-        <f>F94-G94</f>
+        <f t="shared" si="2"/>
         <v>16</v>
       </c>
       <c r="I94" s="7">
-        <f>IF(F94=0,0,H94/F94)</f>
+        <f t="shared" si="3"/>
         <v>6.4935064935064939E-3</v>
       </c>
     </row>
@@ -9688,11 +9685,11 @@
         <v>2358</v>
       </c>
       <c r="H95" s="6">
-        <f>F95-G95</f>
+        <f t="shared" si="2"/>
         <v>16</v>
       </c>
       <c r="I95" s="7">
-        <f>IF(F95=0,0,H95/F95)</f>
+        <f t="shared" si="3"/>
         <v>6.7396798652064023E-3</v>
       </c>
     </row>
@@ -9719,11 +9716,11 @@
         <v>4995</v>
       </c>
       <c r="H96" s="6">
-        <f>F96-G96</f>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
       <c r="I96" s="7">
-        <f>IF(F96=0,0,H96/F96)</f>
+        <f t="shared" si="3"/>
         <v>2.9940119760479044E-3</v>
       </c>
     </row>
@@ -9750,11 +9747,11 @@
         <v>357</v>
       </c>
       <c r="H97" s="6">
-        <f>F97-G97</f>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
       <c r="I97" s="7">
-        <f>IF(F97=0,0,H97/F97)</f>
+        <f t="shared" si="3"/>
         <v>4.0322580645161289E-2</v>
       </c>
     </row>
@@ -9781,11 +9778,11 @@
         <v>2029</v>
       </c>
       <c r="H98" s="6">
-        <f>F98-G98</f>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
       <c r="I98" s="7">
-        <f>IF(F98=0,0,H98/F98)</f>
+        <f t="shared" si="3"/>
         <v>7.3385518590998039E-3</v>
       </c>
     </row>
@@ -9812,11 +9809,11 @@
         <v>490</v>
       </c>
       <c r="H99" s="6">
-        <f>F99-G99</f>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
       <c r="I99" s="7">
-        <f>IF(F99=0,0,H99/F99)</f>
+        <f t="shared" si="3"/>
         <v>2.9702970297029702E-2</v>
       </c>
     </row>
@@ -9843,11 +9840,11 @@
         <v>2254</v>
       </c>
       <c r="H100" s="6">
-        <f>F100-G100</f>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
       <c r="I100" s="7">
-        <f>IF(F100=0,0,H100/F100)</f>
+        <f t="shared" si="3"/>
         <v>6.6108417805200532E-3</v>
       </c>
     </row>
@@ -9874,11 +9871,11 @@
         <v>24740</v>
       </c>
       <c r="H101" s="6">
-        <f>F101-G101</f>
+        <f t="shared" si="2"/>
         <v>14</v>
       </c>
       <c r="I101" s="7">
-        <f>IF(F101=0,0,H101/F101)</f>
+        <f t="shared" si="3"/>
         <v>5.6556516118607097E-4</v>
       </c>
     </row>
@@ -9905,11 +9902,11 @@
         <v>2102</v>
       </c>
       <c r="H102" s="6">
-        <f>F102-G102</f>
+        <f t="shared" si="2"/>
         <v>14</v>
       </c>
       <c r="I102" s="7">
-        <f>IF(F102=0,0,H102/F102)</f>
+        <f t="shared" si="3"/>
         <v>6.6162570888468808E-3</v>
       </c>
     </row>
@@ -9936,11 +9933,11 @@
         <v>21409</v>
       </c>
       <c r="H103" s="6">
-        <f>F103-G103</f>
+        <f t="shared" si="2"/>
         <v>12</v>
       </c>
       <c r="I103" s="7">
-        <f>IF(F103=0,0,H103/F103)</f>
+        <f t="shared" si="3"/>
         <v>5.6019793660426682E-4</v>
       </c>
     </row>
@@ -9967,11 +9964,11 @@
         <v>2668</v>
       </c>
       <c r="H104" s="6">
-        <f>F104-G104</f>
+        <f t="shared" si="2"/>
         <v>12</v>
       </c>
       <c r="I104" s="7">
-        <f>IF(F104=0,0,H104/F104)</f>
+        <f t="shared" si="3"/>
         <v>4.4776119402985077E-3</v>
       </c>
     </row>
@@ -9998,11 +9995,11 @@
         <v>3639.9209999999998</v>
       </c>
       <c r="H105" s="6">
-        <f>F105-G105</f>
+        <f t="shared" si="2"/>
         <v>11.46100000000024</v>
       </c>
       <c r="I105" s="7">
-        <f>IF(F105=0,0,H105/F105)</f>
+        <f t="shared" si="3"/>
         <v>3.138811551352403E-3</v>
       </c>
     </row>
@@ -10029,11 +10026,11 @@
         <v>3558.2820000000002</v>
       </c>
       <c r="H106" s="6">
-        <f>F106-G106</f>
+        <f t="shared" si="2"/>
         <v>11.203999999999724</v>
       </c>
       <c r="I106" s="7">
-        <f>IF(F106=0,0,H106/F106)</f>
+        <f t="shared" si="3"/>
         <v>3.1388272709291266E-3</v>
       </c>
     </row>
@@ -10060,11 +10057,11 @@
         <v>20400</v>
       </c>
       <c r="H107" s="6">
-        <f>F107-G107</f>
+        <f t="shared" si="2"/>
         <v>11</v>
       </c>
       <c r="I107" s="7">
-        <f>IF(F107=0,0,H107/F107)</f>
+        <f t="shared" si="3"/>
         <v>5.3892508941257163E-4</v>
       </c>
     </row>
@@ -10091,11 +10088,11 @@
         <v>18611</v>
       </c>
       <c r="H108" s="6">
-        <f>F108-G108</f>
+        <f t="shared" si="2"/>
         <v>11</v>
       </c>
       <c r="I108" s="7">
-        <f>IF(F108=0,0,H108/F108)</f>
+        <f t="shared" si="3"/>
         <v>5.9069917302115782E-4</v>
       </c>
     </row>
@@ -10122,11 +10119,11 @@
         <v>19806</v>
       </c>
       <c r="H109" s="6">
-        <f>F109-G109</f>
+        <f t="shared" si="2"/>
         <v>11</v>
       </c>
       <c r="I109" s="7">
-        <f>IF(F109=0,0,H109/F109)</f>
+        <f t="shared" si="3"/>
         <v>5.5507897259928342E-4</v>
       </c>
     </row>
@@ -10153,11 +10150,11 @@
         <v>1609</v>
       </c>
       <c r="H110" s="6">
-        <f>F110-G110</f>
+        <f t="shared" si="2"/>
         <v>11</v>
       </c>
       <c r="I110" s="7">
-        <f>IF(F110=0,0,H110/F110)</f>
+        <f t="shared" si="3"/>
         <v>6.7901234567901234E-3</v>
       </c>
     </row>
@@ -10184,11 +10181,11 @@
         <v>3318.9349999999999</v>
       </c>
       <c r="H111" s="6">
-        <f>F111-G111</f>
+        <f t="shared" si="2"/>
         <v>10.450000000000273</v>
       </c>
       <c r="I111" s="7">
-        <f>IF(F111=0,0,H111/F111)</f>
+        <f t="shared" si="3"/>
         <v>3.1387178112475041E-3</v>
       </c>
     </row>
@@ -10215,11 +10212,11 @@
         <v>3309.7080000000001</v>
       </c>
       <c r="H112" s="6">
-        <f>F112-G112</f>
+        <f t="shared" si="2"/>
         <v>10.420999999999822</v>
       </c>
       <c r="I112" s="7">
-        <f>IF(F112=0,0,H112/F112)</f>
+        <f t="shared" si="3"/>
         <v>3.1387334648743533E-3</v>
       </c>
     </row>
@@ -10246,11 +10243,11 @@
         <v>3254.1320000000001</v>
       </c>
       <c r="H113" s="6">
-        <f>F113-G113</f>
+        <f t="shared" si="2"/>
         <v>10.246000000000095</v>
       </c>
       <c r="I113" s="7">
-        <f>IF(F113=0,0,H113/F113)</f>
+        <f t="shared" si="3"/>
         <v>3.1387296446674048E-3</v>
       </c>
     </row>
@@ -10277,11 +10274,11 @@
         <v>3211.6770000000001</v>
       </c>
       <c r="H114" s="6">
-        <f>F114-G114</f>
+        <f t="shared" si="2"/>
         <v>10.11200000000008</v>
       </c>
       <c r="I114" s="7">
-        <f>IF(F114=0,0,H114/F114)</f>
+        <f t="shared" si="3"/>
         <v>3.138628879793208E-3</v>
       </c>
     </row>
@@ -10308,11 +10305,11 @@
         <v>1450</v>
       </c>
       <c r="H115" s="6">
-        <f>F115-G115</f>
+        <f t="shared" si="2"/>
         <v>10</v>
       </c>
       <c r="I115" s="7">
-        <f>IF(F115=0,0,H115/F115)</f>
+        <f t="shared" si="3"/>
         <v>6.8493150684931503E-3</v>
       </c>
     </row>
@@ -10339,11 +10336,11 @@
         <v>1440.9</v>
       </c>
       <c r="H116" s="6">
-        <f>F116-G116</f>
+        <f t="shared" si="2"/>
         <v>10</v>
       </c>
       <c r="I116" s="7">
-        <f>IF(F116=0,0,H116/F116)</f>
+        <f t="shared" si="3"/>
         <v>6.8922737611137909E-3</v>
       </c>
     </row>
@@ -10370,11 +10367,11 @@
         <v>2930.4160000000002</v>
       </c>
       <c r="H117" s="6">
-        <f>F117-G117</f>
+        <f t="shared" si="2"/>
         <v>9.2269999999998618</v>
       </c>
       <c r="I117" s="7">
-        <f>IF(F117=0,0,H117/F117)</f>
+        <f t="shared" si="3"/>
         <v>3.138816516155146E-3</v>
       </c>
     </row>
@@ -10401,11 +10398,11 @@
         <v>16408</v>
       </c>
       <c r="H118" s="6">
-        <f>F118-G118</f>
+        <f t="shared" si="2"/>
         <v>9</v>
       </c>
       <c r="I118" s="7">
-        <f>IF(F118=0,0,H118/F118)</f>
+        <f t="shared" si="3"/>
         <v>5.4821221904123769E-4</v>
       </c>
     </row>
@@ -10432,11 +10429,11 @@
         <v>17339</v>
       </c>
       <c r="H119" s="6">
-        <f>F119-G119</f>
+        <f t="shared" si="2"/>
         <v>9</v>
       </c>
       <c r="I119" s="7">
-        <f>IF(F119=0,0,H119/F119)</f>
+        <f t="shared" si="3"/>
         <v>5.187917915609869E-4</v>
       </c>
     </row>
@@ -10463,11 +10460,11 @@
         <v>1294</v>
       </c>
       <c r="H120" s="6">
-        <f>F120-G120</f>
+        <f t="shared" si="2"/>
         <v>9</v>
       </c>
       <c r="I120" s="7">
-        <f>IF(F120=0,0,H120/F120)</f>
+        <f t="shared" si="3"/>
         <v>6.9071373752877972E-3</v>
       </c>
     </row>
@@ -10494,11 +10491,11 @@
         <v>1329</v>
       </c>
       <c r="H121" s="6">
-        <f>F121-G121</f>
+        <f t="shared" si="2"/>
         <v>9</v>
       </c>
       <c r="I121" s="7">
-        <f>IF(F121=0,0,H121/F121)</f>
+        <f t="shared" si="3"/>
         <v>6.7264573991031393E-3</v>
       </c>
     </row>
@@ -10525,11 +10522,11 @@
         <v>2808.2979999999998</v>
       </c>
       <c r="H122" s="6">
-        <f>F122-G122</f>
+        <f t="shared" si="2"/>
         <v>8.8420000000000982</v>
       </c>
       <c r="I122" s="7">
-        <f>IF(F122=0,0,H122/F122)</f>
+        <f t="shared" si="3"/>
         <v>3.1386441568399506E-3</v>
       </c>
     </row>
@@ -10556,11 +10553,11 @@
         <v>2780.875</v>
       </c>
       <c r="H123" s="6">
-        <f>F123-G123</f>
+        <f t="shared" si="2"/>
         <v>8.7559999999998581</v>
       </c>
       <c r="I123" s="7">
-        <f>IF(F123=0,0,H123/F123)</f>
+        <f t="shared" si="3"/>
         <v>3.1387663816468412E-3</v>
       </c>
     </row>
@@ -10587,11 +10584,11 @@
         <v>2550.422</v>
       </c>
       <c r="H124" s="6">
-        <f>F124-G124</f>
+        <f t="shared" si="2"/>
         <v>8.0300000000002001</v>
       </c>
       <c r="I124" s="7">
-        <f>IF(F124=0,0,H124/F124)</f>
+        <f t="shared" si="3"/>
         <v>3.1386166322448883E-3</v>
       </c>
     </row>
@@ -10618,11 +10615,11 @@
         <v>14197</v>
       </c>
       <c r="H125" s="6">
-        <f>F125-G125</f>
+        <f t="shared" si="2"/>
         <v>8</v>
       </c>
       <c r="I125" s="7">
-        <f>IF(F125=0,0,H125/F125)</f>
+        <f t="shared" si="3"/>
         <v>5.6318197817669833E-4</v>
       </c>
     </row>
@@ -10649,11 +10646,11 @@
         <v>1157</v>
       </c>
       <c r="H126" s="6">
-        <f>F126-G126</f>
+        <f t="shared" si="2"/>
         <v>8</v>
       </c>
       <c r="I126" s="7">
-        <f>IF(F126=0,0,H126/F126)</f>
+        <f t="shared" si="3"/>
         <v>6.8669527896995704E-3</v>
       </c>
     </row>
@@ -10680,11 +10677,11 @@
         <v>1151</v>
       </c>
       <c r="H127" s="6">
-        <f>F127-G127</f>
+        <f t="shared" si="2"/>
         <v>8</v>
       </c>
       <c r="I127" s="7">
-        <f>IF(F127=0,0,H127/F127)</f>
+        <f t="shared" si="3"/>
         <v>6.9025021570319244E-3</v>
       </c>
     </row>
@@ -10711,11 +10708,11 @@
         <v>1198</v>
       </c>
       <c r="H128" s="6">
-        <f>F128-G128</f>
+        <f t="shared" si="2"/>
         <v>8</v>
       </c>
       <c r="I128" s="7">
-        <f>IF(F128=0,0,H128/F128)</f>
+        <f t="shared" si="3"/>
         <v>6.6334991708126038E-3</v>
       </c>
     </row>
@@ -10742,11 +10739,11 @@
         <v>1750</v>
       </c>
       <c r="H129" s="6">
-        <f>F129-G129</f>
+        <f t="shared" si="2"/>
         <v>8</v>
       </c>
       <c r="I129" s="7">
-        <f>IF(F129=0,0,H129/F129)</f>
+        <f t="shared" si="3"/>
         <v>4.5506257110352671E-3</v>
       </c>
     </row>
@@ -10773,11 +10770,11 @@
         <v>1752</v>
       </c>
       <c r="H130" s="6">
-        <f>F130-G130</f>
+        <f t="shared" ref="H130:H193" si="4">F130-G130</f>
         <v>8</v>
       </c>
       <c r="I130" s="7">
-        <f>IF(F130=0,0,H130/F130)</f>
+        <f t="shared" ref="I130:I193" si="5">IF(F130=0,0,H130/F130)</f>
         <v>4.5454545454545452E-3</v>
       </c>
     </row>
@@ -10804,11 +10801,11 @@
         <v>1737</v>
       </c>
       <c r="H131" s="6">
-        <f>F131-G131</f>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
       <c r="I131" s="7">
-        <f>IF(F131=0,0,H131/F131)</f>
+        <f t="shared" si="5"/>
         <v>4.5845272206303722E-3</v>
       </c>
     </row>
@@ -10835,11 +10832,11 @@
         <v>2411.7550000000001</v>
       </c>
       <c r="H132" s="6">
-        <f>F132-G132</f>
+        <f t="shared" si="4"/>
         <v>7.5940000000000509</v>
       </c>
       <c r="I132" s="7">
-        <f>IF(F132=0,0,H132/F132)</f>
+        <f t="shared" si="5"/>
         <v>3.138860908451013E-3</v>
       </c>
     </row>
@@ -10866,11 +10863,11 @@
         <v>11973</v>
       </c>
       <c r="H133" s="6">
-        <f>F133-G133</f>
+        <f t="shared" si="4"/>
         <v>7</v>
       </c>
       <c r="I133" s="7">
-        <f>IF(F133=0,0,H133/F133)</f>
+        <f t="shared" si="5"/>
         <v>5.8430717863105174E-4</v>
       </c>
     </row>
@@ -10897,11 +10894,11 @@
         <v>2073.6669999999999</v>
       </c>
       <c r="H134" s="6">
-        <f>F134-G134</f>
+        <f t="shared" si="4"/>
         <v>6.5289999999999964</v>
       </c>
       <c r="I134" s="7">
-        <f>IF(F134=0,0,H134/F134)</f>
+        <f t="shared" si="5"/>
         <v>3.1386465506134981E-3</v>
       </c>
     </row>
@@ -10928,11 +10925,11 @@
         <v>2019.0809999999999</v>
       </c>
       <c r="H135" s="6">
-        <f>F135-G135</f>
+        <f t="shared" si="4"/>
         <v>6.3570000000001983</v>
       </c>
       <c r="I135" s="7">
-        <f>IF(F135=0,0,H135/F135)</f>
+        <f t="shared" si="5"/>
         <v>3.1385803959440863E-3</v>
       </c>
     </row>
@@ -10959,11 +10956,11 @@
         <v>1986.462</v>
       </c>
       <c r="H136" s="6">
-        <f>F136-G136</f>
+        <f t="shared" si="4"/>
         <v>6.2550000000001091</v>
       </c>
       <c r="I136" s="7">
-        <f>IF(F136=0,0,H136/F136)</f>
+        <f t="shared" si="5"/>
         <v>3.1389304151066655E-3</v>
       </c>
     </row>
@@ -10990,11 +10987,11 @@
         <v>1919.5350000000001</v>
       </c>
       <c r="H137" s="6">
-        <f>F137-G137</f>
+        <f t="shared" si="4"/>
         <v>6.043999999999869</v>
       </c>
       <c r="I137" s="7">
-        <f>IF(F137=0,0,H137/F137)</f>
+        <f t="shared" si="5"/>
         <v>3.1387961750724688E-3</v>
       </c>
     </row>
@@ -11021,11 +11018,11 @@
         <v>10380</v>
       </c>
       <c r="H138" s="6">
-        <f>F138-G138</f>
+        <f t="shared" si="4"/>
         <v>6</v>
       </c>
       <c r="I138" s="7">
-        <f>IF(F138=0,0,H138/F138)</f>
+        <f t="shared" si="5"/>
         <v>5.7770075101097628E-4</v>
       </c>
     </row>
@@ -11052,11 +11049,11 @@
         <v>1414</v>
       </c>
       <c r="H139" s="6">
-        <f>F139-G139</f>
+        <f t="shared" si="4"/>
         <v>6</v>
       </c>
       <c r="I139" s="7">
-        <f>IF(F139=0,0,H139/F139)</f>
+        <f t="shared" si="5"/>
         <v>4.2253521126760559E-3</v>
       </c>
     </row>
@@ -11083,11 +11080,11 @@
         <v>1894.866</v>
       </c>
       <c r="H140" s="6">
-        <f>F140-G140</f>
+        <f t="shared" si="4"/>
         <v>5.9660000000001219</v>
       </c>
       <c r="I140" s="7">
-        <f>IF(F140=0,0,H140/F140)</f>
+        <f t="shared" si="5"/>
         <v>3.1386256123634923E-3</v>
       </c>
     </row>
@@ -11114,11 +11111,11 @@
         <v>1692.5250000000001</v>
       </c>
       <c r="H141" s="6">
-        <f>F141-G141</f>
+        <f t="shared" si="4"/>
         <v>5.3289999999999509</v>
       </c>
       <c r="I141" s="7">
-        <f>IF(F141=0,0,H141/F141)</f>
+        <f t="shared" si="5"/>
         <v>3.1386679891203546E-3</v>
       </c>
     </row>
@@ -11145,11 +11142,11 @@
         <v>1613.9780000000001</v>
       </c>
       <c r="H142" s="6">
-        <f>F142-G142</f>
+        <f t="shared" si="4"/>
         <v>5.0819999999998799</v>
       </c>
       <c r="I142" s="7">
-        <f>IF(F142=0,0,H142/F142)</f>
+        <f t="shared" si="5"/>
         <v>3.1388583499066618E-3</v>
       </c>
     </row>
@@ -11176,11 +11173,11 @@
         <v>8741</v>
       </c>
       <c r="H143" s="6">
-        <f>F143-G143</f>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="I143" s="7">
-        <f>IF(F143=0,0,H143/F143)</f>
+        <f t="shared" si="5"/>
         <v>5.7168991538989247E-4</v>
       </c>
     </row>
@@ -11207,11 +11204,11 @@
         <v>8233</v>
       </c>
       <c r="H144" s="6">
-        <f>F144-G144</f>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="I144" s="7">
-        <f>IF(F144=0,0,H144/F144)</f>
+        <f t="shared" si="5"/>
         <v>6.0694343287205632E-4</v>
       </c>
     </row>
@@ -11238,11 +11235,11 @@
         <v>9474</v>
       </c>
       <c r="H145" s="6">
-        <f>F145-G145</f>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="I145" s="7">
-        <f>IF(F145=0,0,H145/F145)</f>
+        <f t="shared" si="5"/>
         <v>5.2748180187783518E-4</v>
       </c>
     </row>
@@ -11269,11 +11266,11 @@
         <v>229</v>
       </c>
       <c r="H146" s="6">
-        <f>F146-G146</f>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="I146" s="7">
-        <f>IF(F146=0,0,H146/F146)</f>
+        <f t="shared" si="5"/>
         <v>2.1367521367521368E-2</v>
       </c>
     </row>
@@ -11300,11 +11297,11 @@
         <v>1144</v>
       </c>
       <c r="H147" s="6">
-        <f>F147-G147</f>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="I147" s="7">
-        <f>IF(F147=0,0,H147/F147)</f>
+        <f t="shared" si="5"/>
         <v>4.3516100957354219E-3</v>
       </c>
     </row>
@@ -11331,11 +11328,11 @@
         <v>1152</v>
       </c>
       <c r="H148" s="6">
-        <f>F148-G148</f>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="I148" s="7">
-        <f>IF(F148=0,0,H148/F148)</f>
+        <f t="shared" si="5"/>
         <v>4.3215211754537601E-3</v>
       </c>
     </row>
@@ -11362,11 +11359,11 @@
         <v>1400.9179999999999</v>
       </c>
       <c r="H149" s="6">
-        <f>F149-G149</f>
+        <f t="shared" si="4"/>
         <v>4.4110000000000582</v>
       </c>
       <c r="I149" s="7">
-        <f>IF(F149=0,0,H149/F149)</f>
+        <f t="shared" si="5"/>
         <v>3.1387667941101751E-3</v>
       </c>
     </row>
@@ -11393,11 +11390,11 @@
         <v>609</v>
       </c>
       <c r="H150" s="6">
-        <f>F150-G150</f>
+        <f t="shared" si="4"/>
         <v>4</v>
       </c>
       <c r="I150" s="7">
-        <f>IF(F150=0,0,H150/F150)</f>
+        <f t="shared" si="5"/>
         <v>6.5252854812398045E-3</v>
       </c>
     </row>
@@ -11424,11 +11421,11 @@
         <v>623</v>
       </c>
       <c r="H151" s="6">
-        <f>F151-G151</f>
+        <f t="shared" si="4"/>
         <v>4</v>
       </c>
       <c r="I151" s="7">
-        <f>IF(F151=0,0,H151/F151)</f>
+        <f t="shared" si="5"/>
         <v>6.379585326953748E-3</v>
       </c>
     </row>
@@ -11455,11 +11452,11 @@
         <v>1002</v>
       </c>
       <c r="H152" s="6">
-        <f>F152-G152</f>
+        <f t="shared" si="4"/>
         <v>4</v>
       </c>
       <c r="I152" s="7">
-        <f>IF(F152=0,0,H152/F152)</f>
+        <f t="shared" si="5"/>
         <v>3.9761431411530811E-3</v>
       </c>
     </row>
@@ -11486,11 +11483,11 @@
         <v>1089.8309999999999</v>
       </c>
       <c r="H153" s="6">
-        <f>F153-G153</f>
+        <f t="shared" si="4"/>
         <v>3.43100000000004</v>
       </c>
       <c r="I153" s="7">
-        <f>IF(F153=0,0,H153/F153)</f>
+        <f t="shared" si="5"/>
         <v>3.1383145119834406E-3</v>
       </c>
     </row>
@@ -11517,11 +11514,11 @@
         <v>5781</v>
       </c>
       <c r="H154" s="6">
-        <f>F154-G154</f>
+        <f t="shared" si="4"/>
         <v>3</v>
       </c>
       <c r="I154" s="7">
-        <f>IF(F154=0,0,H154/F154)</f>
+        <f t="shared" si="5"/>
         <v>5.1867219917012448E-4</v>
       </c>
     </row>
@@ -11548,11 +11545,11 @@
         <v>5782</v>
       </c>
       <c r="H155" s="6">
-        <f>F155-G155</f>
+        <f t="shared" si="4"/>
         <v>3</v>
       </c>
       <c r="I155" s="7">
-        <f>IF(F155=0,0,H155/F155)</f>
+        <f t="shared" si="5"/>
         <v>5.185825410544512E-4</v>
       </c>
     </row>
@@ -11579,11 +11576,11 @@
         <v>3977</v>
       </c>
       <c r="H156" s="6">
-        <f>F156-G156</f>
+        <f t="shared" si="4"/>
         <v>3</v>
       </c>
       <c r="I156" s="7">
-        <f>IF(F156=0,0,H156/F156)</f>
+        <f t="shared" si="5"/>
         <v>7.537688442211055E-4</v>
       </c>
     </row>
@@ -11610,11 +11607,11 @@
         <v>436.3</v>
       </c>
       <c r="H157" s="6">
-        <f>F157-G157</f>
+        <f t="shared" si="4"/>
         <v>3</v>
       </c>
       <c r="I157" s="7">
-        <f>IF(F157=0,0,H157/F157)</f>
+        <f t="shared" si="5"/>
         <v>6.8290462098793536E-3</v>
       </c>
     </row>
@@ -11641,11 +11638,11 @@
         <v>419</v>
       </c>
       <c r="H158" s="6">
-        <f>F158-G158</f>
+        <f t="shared" si="4"/>
         <v>3</v>
       </c>
       <c r="I158" s="7">
-        <f>IF(F158=0,0,H158/F158)</f>
+        <f t="shared" si="5"/>
         <v>7.1090047393364926E-3</v>
       </c>
     </row>
@@ -11672,11 +11669,11 @@
         <v>377</v>
       </c>
       <c r="H159" s="6">
-        <f>F159-G159</f>
+        <f t="shared" si="4"/>
         <v>3</v>
       </c>
       <c r="I159" s="7">
-        <f>IF(F159=0,0,H159/F159)</f>
+        <f t="shared" si="5"/>
         <v>7.8947368421052634E-3</v>
       </c>
     </row>
@@ -11703,11 +11700,11 @@
         <v>417</v>
       </c>
       <c r="H160" s="6">
-        <f>F160-G160</f>
+        <f t="shared" si="4"/>
         <v>3</v>
       </c>
       <c r="I160" s="7">
-        <f>IF(F160=0,0,H160/F160)</f>
+        <f t="shared" si="5"/>
         <v>7.1428571428571426E-3</v>
       </c>
     </row>
@@ -11734,11 +11731,11 @@
         <v>839</v>
       </c>
       <c r="H161" s="6">
-        <f>F161-G161</f>
+        <f t="shared" si="4"/>
         <v>3</v>
       </c>
       <c r="I161" s="7">
-        <f>IF(F161=0,0,H161/F161)</f>
+        <f t="shared" si="5"/>
         <v>3.5629453681710215E-3</v>
       </c>
     </row>
@@ -11765,11 +11762,11 @@
         <v>617</v>
       </c>
       <c r="H162" s="6">
-        <f>F162-G162</f>
+        <f t="shared" si="4"/>
         <v>3</v>
       </c>
       <c r="I162" s="7">
-        <f>IF(F162=0,0,H162/F162)</f>
+        <f t="shared" si="5"/>
         <v>4.8387096774193551E-3</v>
       </c>
     </row>
@@ -11796,11 +11793,11 @@
         <v>703.92100000000005</v>
       </c>
       <c r="H163" s="6">
-        <f>F163-G163</f>
+        <f t="shared" si="4"/>
         <v>2.2159999999998945</v>
       </c>
       <c r="I163" s="7">
-        <f>IF(F163=0,0,H163/F163)</f>
+        <f t="shared" si="5"/>
         <v>3.1382012272404571E-3</v>
       </c>
     </row>
@@ -11827,11 +11824,11 @@
         <v>2757</v>
       </c>
       <c r="H164" s="6">
-        <f>F164-G164</f>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="I164" s="7">
-        <f>IF(F164=0,0,H164/F164)</f>
+        <f t="shared" si="5"/>
         <v>7.2490032620514677E-4</v>
       </c>
     </row>
@@ -11858,11 +11855,11 @@
         <v>1931</v>
       </c>
       <c r="H165" s="6">
-        <f>F165-G165</f>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="I165" s="7">
-        <f>IF(F165=0,0,H165/F165)</f>
+        <f t="shared" si="5"/>
         <v>1.0346611484738748E-3</v>
       </c>
     </row>
@@ -11889,11 +11886,11 @@
         <v>328</v>
       </c>
       <c r="H166" s="6">
-        <f>F166-G166</f>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="I166" s="7">
-        <f>IF(F166=0,0,H166/F166)</f>
+        <f t="shared" si="5"/>
         <v>6.0606060606060606E-3</v>
       </c>
     </row>
@@ -11920,11 +11917,11 @@
         <v>328</v>
       </c>
       <c r="H167" s="6">
-        <f>F167-G167</f>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="I167" s="7">
-        <f>IF(F167=0,0,H167/F167)</f>
+        <f t="shared" si="5"/>
         <v>6.0606060606060606E-3</v>
       </c>
     </row>
@@ -11951,11 +11948,11 @@
         <v>376</v>
       </c>
       <c r="H168" s="6">
-        <f>F168-G168</f>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="I168" s="7">
-        <f>IF(F168=0,0,H168/F168)</f>
+        <f t="shared" si="5"/>
         <v>5.2910052910052907E-3</v>
       </c>
     </row>
@@ -11982,11 +11979,11 @@
         <v>395</v>
       </c>
       <c r="H169" s="6">
-        <f>F169-G169</f>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="I169" s="7">
-        <f>IF(F169=0,0,H169/F169)</f>
+        <f t="shared" si="5"/>
         <v>5.0377833753148613E-3</v>
       </c>
     </row>
@@ -12013,11 +12010,11 @@
         <v>454</v>
       </c>
       <c r="H170" s="6">
-        <f>F170-G170</f>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="I170" s="7">
-        <f>IF(F170=0,0,H170/F170)</f>
+        <f t="shared" si="5"/>
         <v>4.3859649122807015E-3</v>
       </c>
     </row>
@@ -12044,11 +12041,11 @@
         <v>400</v>
       </c>
       <c r="H171" s="6">
-        <f>F171-G171</f>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="I171" s="7">
-        <f>IF(F171=0,0,H171/F171)</f>
+        <f t="shared" si="5"/>
         <v>4.9751243781094526E-3</v>
       </c>
     </row>
@@ -12075,11 +12072,11 @@
         <v>566</v>
       </c>
       <c r="H172" s="6">
-        <f>F172-G172</f>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="I172" s="7">
-        <f>IF(F172=0,0,H172/F172)</f>
+        <f t="shared" si="5"/>
         <v>3.5211267605633804E-3</v>
       </c>
     </row>
@@ -12106,11 +12103,11 @@
         <v>425</v>
       </c>
       <c r="H173" s="6">
-        <f>F173-G173</f>
+        <f t="shared" si="4"/>
         <v>2</v>
       </c>
       <c r="I173" s="7">
-        <f>IF(F173=0,0,H173/F173)</f>
+        <f t="shared" si="5"/>
         <v>4.6838407494145199E-3</v>
       </c>
     </row>
@@ -12137,11 +12134,11 @@
         <v>634.096</v>
       </c>
       <c r="H174" s="6">
-        <f>F174-G174</f>
+        <f t="shared" si="4"/>
         <v>1.9969999999999573</v>
       </c>
       <c r="I174" s="7">
-        <f>IF(F174=0,0,H174/F174)</f>
+        <f t="shared" si="5"/>
         <v>3.1394780323002413E-3</v>
       </c>
     </row>
@@ -12168,11 +12165,11 @@
         <v>611.38800000000003</v>
       </c>
       <c r="H175" s="6">
-        <f>F175-G175</f>
+        <f t="shared" si="4"/>
         <v>1.9249999999999545</v>
       </c>
       <c r="I175" s="7">
-        <f>IF(F175=0,0,H175/F175)</f>
+        <f t="shared" si="5"/>
         <v>3.1386910109519194E-3</v>
       </c>
     </row>
@@ -12199,11 +12196,11 @@
         <v>457.37900000000002</v>
       </c>
       <c r="H176" s="6">
-        <f>F176-G176</f>
+        <f t="shared" si="4"/>
         <v>1.4399999999999977</v>
       </c>
       <c r="I176" s="7">
-        <f>IF(F176=0,0,H176/F176)</f>
+        <f t="shared" si="5"/>
         <v>3.1384925210159076E-3</v>
       </c>
     </row>
@@ -12230,11 +12227,11 @@
         <v>408.35199999999998</v>
       </c>
       <c r="H177" s="6">
-        <f>F177-G177</f>
+        <f t="shared" si="4"/>
         <v>1.2860000000000014</v>
       </c>
       <c r="I177" s="7">
-        <f>IF(F177=0,0,H177/F177)</f>
+        <f t="shared" si="5"/>
         <v>3.1393571885420823E-3</v>
       </c>
     </row>
@@ -12261,11 +12258,11 @@
         <v>1792</v>
       </c>
       <c r="H178" s="6">
-        <f>F178-G178</f>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="I178" s="7">
-        <f>IF(F178=0,0,H178/F178)</f>
+        <f t="shared" si="5"/>
         <v>5.5772448410485224E-4</v>
       </c>
     </row>
@@ -12292,11 +12289,11 @@
         <v>2272</v>
       </c>
       <c r="H179" s="6">
-        <f>F179-G179</f>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="I179" s="7">
-        <f>IF(F179=0,0,H179/F179)</f>
+        <f t="shared" si="5"/>
         <v>4.399472063352398E-4</v>
       </c>
     </row>
@@ -12323,11 +12320,11 @@
         <v>2101</v>
       </c>
       <c r="H180" s="6">
-        <f>F180-G180</f>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="I180" s="7">
-        <f>IF(F180=0,0,H180/F180)</f>
+        <f t="shared" si="5"/>
         <v>4.7573739295908661E-4</v>
       </c>
     </row>
@@ -12354,11 +12351,11 @@
         <v>937</v>
       </c>
       <c r="H181" s="6">
-        <f>F181-G181</f>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="I181" s="7">
-        <f>IF(F181=0,0,H181/F181)</f>
+        <f t="shared" si="5"/>
         <v>1.0660980810234541E-3</v>
       </c>
     </row>
@@ -12385,11 +12382,11 @@
         <v>774</v>
       </c>
       <c r="H182" s="6">
-        <f>F182-G182</f>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="I182" s="7">
-        <f>IF(F182=0,0,H182/F182)</f>
+        <f t="shared" si="5"/>
         <v>1.2903225806451613E-3</v>
       </c>
     </row>
@@ -12416,11 +12413,11 @@
         <v>2957</v>
       </c>
       <c r="H183" s="6">
-        <f>F183-G183</f>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="I183" s="7">
-        <f>IF(F183=0,0,H183/F183)</f>
+        <f t="shared" si="5"/>
         <v>3.3806626098715348E-4</v>
       </c>
     </row>
@@ -12447,11 +12444,11 @@
         <v>407</v>
       </c>
       <c r="H184" s="6">
-        <f>F184-G184</f>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="I184" s="7">
-        <f>IF(F184=0,0,H184/F184)</f>
+        <f t="shared" si="5"/>
         <v>2.4509803921568627E-3</v>
       </c>
     </row>
@@ -12478,11 +12475,11 @@
         <v>3167</v>
       </c>
       <c r="H185" s="6">
-        <f>F185-G185</f>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="I185" s="7">
-        <f>IF(F185=0,0,H185/F185)</f>
+        <f t="shared" si="5"/>
         <v>3.1565656565656568E-4</v>
       </c>
     </row>
@@ -12509,11 +12506,11 @@
         <v>125</v>
       </c>
       <c r="H186" s="6">
-        <f>F186-G186</f>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="I186" s="7">
-        <f>IF(F186=0,0,H186/F186)</f>
+        <f t="shared" si="5"/>
         <v>7.9365079365079361E-3</v>
       </c>
     </row>
@@ -12540,11 +12537,11 @@
         <v>207</v>
       </c>
       <c r="H187" s="6">
-        <f>F187-G187</f>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="I187" s="7">
-        <f>IF(F187=0,0,H187/F187)</f>
+        <f t="shared" si="5"/>
         <v>4.807692307692308E-3</v>
       </c>
     </row>
@@ -12571,11 +12568,11 @@
         <v>224</v>
       </c>
       <c r="H188" s="6">
-        <f>F188-G188</f>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="I188" s="7">
-        <f>IF(F188=0,0,H188/F188)</f>
+        <f t="shared" si="5"/>
         <v>4.4444444444444444E-3</v>
       </c>
     </row>
@@ -12602,11 +12599,11 @@
         <v>151</v>
       </c>
       <c r="H189" s="6">
-        <f>F189-G189</f>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="I189" s="7">
-        <f>IF(F189=0,0,H189/F189)</f>
+        <f t="shared" si="5"/>
         <v>6.5789473684210523E-3</v>
       </c>
     </row>
@@ -12633,11 +12630,11 @@
         <v>295</v>
       </c>
       <c r="H190" s="6">
-        <f>F190-G190</f>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="I190" s="7">
-        <f>IF(F190=0,0,H190/F190)</f>
+        <f t="shared" si="5"/>
         <v>3.3783783783783786E-3</v>
       </c>
     </row>
@@ -12664,11 +12661,11 @@
         <v>244</v>
       </c>
       <c r="H191" s="6">
-        <f>F191-G191</f>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="I191" s="7">
-        <f>IF(F191=0,0,H191/F191)</f>
+        <f t="shared" si="5"/>
         <v>4.0816326530612249E-3</v>
       </c>
     </row>
@@ -12695,11 +12692,11 @@
         <v>218</v>
       </c>
       <c r="H192" s="6">
-        <f>F192-G192</f>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="I192" s="7">
-        <f>IF(F192=0,0,H192/F192)</f>
+        <f t="shared" si="5"/>
         <v>4.5662100456621002E-3</v>
       </c>
     </row>
@@ -12726,11 +12723,11 @@
         <v>233</v>
       </c>
       <c r="H193" s="6">
-        <f>F193-G193</f>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="I193" s="7">
-        <f>IF(F193=0,0,H193/F193)</f>
+        <f t="shared" si="5"/>
         <v>4.2735042735042739E-3</v>
       </c>
     </row>
@@ -12757,11 +12754,11 @@
         <v>288</v>
       </c>
       <c r="H194" s="6">
-        <f>F194-G194</f>
+        <f t="shared" ref="H194:H257" si="6">F194-G194</f>
         <v>1</v>
       </c>
       <c r="I194" s="7">
-        <f>IF(F194=0,0,H194/F194)</f>
+        <f t="shared" ref="I194:I257" si="7">IF(F194=0,0,H194/F194)</f>
         <v>3.4602076124567475E-3</v>
       </c>
     </row>
@@ -12788,11 +12785,11 @@
         <v>285</v>
       </c>
       <c r="H195" s="6">
-        <f>F195-G195</f>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="I195" s="7">
-        <f>IF(F195=0,0,H195/F195)</f>
+        <f t="shared" si="7"/>
         <v>3.4965034965034965E-3</v>
       </c>
     </row>
@@ -12819,11 +12816,11 @@
         <v>319</v>
       </c>
       <c r="H196" s="6">
-        <f>F196-G196</f>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="I196" s="7">
-        <f>IF(F196=0,0,H196/F196)</f>
+        <f t="shared" si="7"/>
         <v>3.1250000000000002E-3</v>
       </c>
     </row>
@@ -12850,11 +12847,11 @@
         <v>178</v>
       </c>
       <c r="H197" s="6">
-        <f>F197-G197</f>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="I197" s="7">
-        <f>IF(F197=0,0,H197/F197)</f>
+        <f t="shared" si="7"/>
         <v>5.5865921787709499E-3</v>
       </c>
     </row>
@@ -12881,11 +12878,11 @@
         <v>330</v>
       </c>
       <c r="H198" s="6">
-        <f>F198-G198</f>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="I198" s="7">
-        <f>IF(F198=0,0,H198/F198)</f>
+        <f t="shared" si="7"/>
         <v>3.0211480362537764E-3</v>
       </c>
     </row>
@@ -12912,11 +12909,11 @@
         <v>147</v>
       </c>
       <c r="H199" s="6">
-        <f>F199-G199</f>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="I199" s="7">
-        <f>IF(F199=0,0,H199/F199)</f>
+        <f t="shared" si="7"/>
         <v>6.7567567567567571E-3</v>
       </c>
     </row>
@@ -12943,11 +12940,11 @@
         <v>285</v>
       </c>
       <c r="H200" s="6">
-        <f>F200-G200</f>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="I200" s="7">
-        <f>IF(F200=0,0,H200/F200)</f>
+        <f t="shared" si="7"/>
         <v>3.4965034965034965E-3</v>
       </c>
     </row>
@@ -12974,11 +12971,11 @@
         <v>248</v>
       </c>
       <c r="H201" s="6">
-        <f>F201-G201</f>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="I201" s="7">
-        <f>IF(F201=0,0,H201/F201)</f>
+        <f t="shared" si="7"/>
         <v>4.0160642570281121E-3</v>
       </c>
     </row>
@@ -13005,11 +13002,11 @@
         <v>223</v>
       </c>
       <c r="H202" s="6">
-        <f>F202-G202</f>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="I202" s="7">
-        <f>IF(F202=0,0,H202/F202)</f>
+        <f t="shared" si="7"/>
         <v>4.464285714285714E-3</v>
       </c>
     </row>
@@ -13036,11 +13033,11 @@
         <v>253</v>
       </c>
       <c r="H203" s="6">
-        <f>F203-G203</f>
+        <f t="shared" si="6"/>
         <v>1</v>
       </c>
       <c r="I203" s="7">
-        <f>IF(F203=0,0,H203/F203)</f>
+        <f t="shared" si="7"/>
         <v>3.937007874015748E-3</v>
       </c>
     </row>
@@ -13067,11 +13064,11 @@
         <v>280.90800000000002</v>
       </c>
       <c r="H204" s="6">
-        <f>F204-G204</f>
+        <f t="shared" si="6"/>
         <v>0.88399999999995771</v>
       </c>
       <c r="I204" s="7">
-        <f>IF(F204=0,0,H204/F204)</f>
+        <f t="shared" si="7"/>
         <v>3.1370656370654872E-3</v>
       </c>
     </row>
@@ -13098,11 +13095,11 @@
         <v>186.03800000000001</v>
       </c>
       <c r="H205" s="6">
-        <f>F205-G205</f>
+        <f t="shared" si="6"/>
         <v>0.58599999999998431</v>
       </c>
       <c r="I205" s="7">
-        <f>IF(F205=0,0,H205/F205)</f>
+        <f t="shared" si="7"/>
         <v>3.1400034293551974E-3</v>
       </c>
     </row>
@@ -13129,11 +13126,11 @@
         <v>157.57900000000001</v>
       </c>
       <c r="H206" s="6">
-        <f>F206-G206</f>
+        <f t="shared" si="6"/>
         <v>0.4959999999999809</v>
       </c>
       <c r="I206" s="7">
-        <f>IF(F206=0,0,H206/F206)</f>
+        <f t="shared" si="7"/>
         <v>3.1377510675311146E-3</v>
       </c>
     </row>
@@ -13160,11 +13157,11 @@
         <v>97.022000000000006</v>
       </c>
       <c r="H207" s="6">
-        <f>F207-G207</f>
+        <f t="shared" si="6"/>
         <v>0.30499999999999261</v>
       </c>
       <c r="I207" s="7">
-        <f>IF(F207=0,0,H207/F207)</f>
+        <f t="shared" si="7"/>
         <v>3.1337655532379773E-3</v>
       </c>
     </row>

</xml_diff>